<commit_message>
Tracker v1.2 and Week 1-2 lessons: map tasks to ReadyForProd lectures
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tracker/75-Day-Career-Upgrade-Tracker.xlsx
+++ b/tracker/75-Day-Career-Upgrade-Tracker.xlsx
@@ -15,7 +15,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Projects" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Daily'!$A$1:$I$80</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Daily'!$A$1:$J$80</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -65,12 +65,12 @@
       <sz val="11"/>
     </font>
     <font>
+      <i val="1"/>
+      <color rgb="005B6B78"/>
+    </font>
+    <font>
       <b val="1"/>
       <color rgb="0017324D"/>
-    </font>
-    <font>
-      <i val="1"/>
-      <color rgb="005B6B78"/>
     </font>
     <font>
       <b val="1"/>
@@ -142,7 +142,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -173,14 +173,17 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -579,7 +582,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:C32"/>
+  <dimension ref="B2:C33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -792,25 +795,29 @@
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="B27" s="5" t="inlineStr">
+    <row r="26">
+      <c r="B26" s="6" t="inlineStr">
+        <is>
+          <t>Courses in the Daily tab</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>Optional. Every task can be done with the free resource. Already own one of these courses on Udemy? Use it there, the topic is the same.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" s="5" t="inlineStr">
         <is>
           <t>My goal</t>
         </is>
       </c>
-    </row>
-    <row r="28">
-      <c r="B28" s="6" t="inlineStr">
-        <is>
-          <t>In 75 days I want to be able to…</t>
-        </is>
-      </c>
-      <c r="C28" s="8" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="B29" s="6" t="inlineStr">
         <is>
-          <t>…so that…</t>
+          <t>In 75 days I want to be able to…</t>
         </is>
       </c>
       <c r="C29" s="8" t="inlineStr"/>
@@ -818,20 +825,28 @@
     <row r="30">
       <c r="B30" s="6" t="inlineStr">
         <is>
+          <t>…so that…</t>
+        </is>
+      </c>
+      <c r="C30" s="8" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="B31" s="6" t="inlineStr">
+        <is>
           <t>My Day 1 date</t>
         </is>
       </c>
-      <c r="C30" s="8" t="inlineStr"/>
-    </row>
-    <row r="32">
-      <c r="B32" s="6" t="inlineStr">
+      <c r="C31" s="8" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="B33" s="6" t="inlineStr">
         <is>
           <t>Tracker version</t>
         </is>
       </c>
-      <c r="C32" s="4" t="inlineStr">
-        <is>
-          <t>v1.1 (Oct 2026). Content lives in the weekly lessons, so it updates without downloading again.</t>
+      <c r="C33" s="4" t="inlineStr">
+        <is>
+          <t>v1.2 (Oct 2026). Content lives in the weekly lessons, so it updates without downloading again.</t>
         </is>
       </c>
     </row>
@@ -877,7 +892,7 @@
         </is>
       </c>
       <c r="C2" s="11">
-        <f>COUNTIFS(Daily!A6:A80,"&gt;=1",Daily!G6:G80,"Yes")</f>
+        <f>COUNTIFS(Daily!A6:A80,"&gt;=1",Daily!H6:H80,"Yes")</f>
         <v/>
       </c>
     </row>
@@ -888,7 +903,7 @@
         </is>
       </c>
       <c r="C3" s="11">
-        <f>COUNTIF(Daily!G6:G80,"Partly")</f>
+        <f>COUNTIF(Daily!H6:H80,"Partly")</f>
         <v/>
       </c>
     </row>
@@ -910,7 +925,7 @@
         </is>
       </c>
       <c r="C5" s="11">
-        <f>SUM(Daily!H2:H80)</f>
+        <f>SUM(Daily!I2:I80)</f>
         <v/>
       </c>
     </row>
@@ -961,7 +976,7 @@
         </is>
       </c>
       <c r="C11">
-        <f>COUNTIFS(Daily!B6:B80,1,Daily!G6:G80,"Yes")</f>
+        <f>COUNTIFS(Daily!B6:B80,1,Daily!H6:H80,"Yes")</f>
         <v/>
       </c>
     </row>
@@ -972,7 +987,7 @@
         </is>
       </c>
       <c r="C12">
-        <f>COUNTIFS(Daily!B6:B80,2,Daily!G6:G80,"Yes")</f>
+        <f>COUNTIFS(Daily!B6:B80,2,Daily!H6:H80,"Yes")</f>
         <v/>
       </c>
     </row>
@@ -983,7 +998,7 @@
         </is>
       </c>
       <c r="C13">
-        <f>COUNTIFS(Daily!B6:B80,3,Daily!G6:G80,"Yes")</f>
+        <f>COUNTIFS(Daily!B6:B80,3,Daily!H6:H80,"Yes")</f>
         <v/>
       </c>
     </row>
@@ -994,7 +1009,7 @@
         </is>
       </c>
       <c r="C14">
-        <f>COUNTIFS(Daily!B6:B80,4,Daily!G6:G80,"Yes")</f>
+        <f>COUNTIFS(Daily!B6:B80,4,Daily!H6:H80,"Yes")</f>
         <v/>
       </c>
     </row>
@@ -1005,7 +1020,7 @@
         </is>
       </c>
       <c r="C15">
-        <f>COUNTIFS(Daily!B6:B80,5,Daily!G6:G80,"Yes")</f>
+        <f>COUNTIFS(Daily!B6:B80,5,Daily!H6:H80,"Yes")</f>
         <v/>
       </c>
     </row>
@@ -1016,7 +1031,7 @@
         </is>
       </c>
       <c r="C16">
-        <f>COUNTIFS(Daily!B6:B80,6,Daily!G6:G80,"Yes")</f>
+        <f>COUNTIFS(Daily!B6:B80,6,Daily!H6:H80,"Yes")</f>
         <v/>
       </c>
     </row>
@@ -1027,7 +1042,7 @@
         </is>
       </c>
       <c r="C17">
-        <f>COUNTIFS(Daily!B6:B80,7,Daily!G6:G80,"Yes")</f>
+        <f>COUNTIFS(Daily!B6:B80,7,Daily!H6:H80,"Yes")</f>
         <v/>
       </c>
     </row>
@@ -1038,7 +1053,7 @@
         </is>
       </c>
       <c r="C18">
-        <f>COUNTIFS(Daily!B6:B80,8,Daily!G6:G80,"Yes")</f>
+        <f>COUNTIFS(Daily!B6:B80,8,Daily!H6:H80,"Yes")</f>
         <v/>
       </c>
     </row>
@@ -1049,7 +1064,7 @@
         </is>
       </c>
       <c r="C19">
-        <f>COUNTIFS(Daily!B6:B80,9,Daily!G6:G80,"Yes")</f>
+        <f>COUNTIFS(Daily!B6:B80,9,Daily!H6:H80,"Yes")</f>
         <v/>
       </c>
     </row>
@@ -1060,7 +1075,7 @@
         </is>
       </c>
       <c r="C20">
-        <f>COUNTIFS(Daily!B6:B80,10,Daily!G6:G80,"Yes")</f>
+        <f>COUNTIFS(Daily!B6:B80,10,Daily!H6:H80,"Yes")</f>
         <v/>
       </c>
     </row>
@@ -1071,7 +1086,7 @@
         </is>
       </c>
       <c r="C21">
-        <f>COUNTIFS(Daily!B6:B80,11,Daily!G6:G80,"Yes")</f>
+        <f>COUNTIFS(Daily!B6:B80,11,Daily!H6:H80,"Yes")</f>
         <v/>
       </c>
     </row>
@@ -1086,7 +1101,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I80"/>
+  <dimension ref="A1:J80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1095,9 +1110,10 @@
     <col width="26" customWidth="1" min="4" max="4"/>
     <col width="70" customWidth="1" min="5" max="5"/>
     <col width="38" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="9" customWidth="1" min="8" max="8"/>
-    <col width="45" customWidth="1" min="9" max="9"/>
+    <col width="42" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="9" customWidth="1" min="9" max="9"/>
+    <col width="45" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -1128,20 +1144,25 @@
       </c>
       <c r="F1" s="13" t="inlineStr">
         <is>
-          <t>Resource</t>
+          <t>Free resource</t>
         </is>
       </c>
       <c r="G1" s="13" t="inlineStr">
         <is>
+          <t>In our courses (optional, faster)</t>
+        </is>
+      </c>
+      <c r="H1" s="13" t="inlineStr">
+        <is>
           <t>Done?</t>
         </is>
       </c>
-      <c r="H1" s="13" t="inlineStr">
+      <c r="I1" s="13" t="inlineStr">
         <is>
           <t>Minutes</t>
         </is>
       </c>
-      <c r="I1" s="13" t="inlineStr">
+      <c r="J1" s="13" t="inlineStr">
         <is>
           <t>My notes (what worked, what didn't)</t>
         </is>
@@ -1176,9 +1197,10 @@
           <t>https://github.com/TechSckoolByVijay/75-day-career-upgrade/tree/main/week-00-setup</t>
         </is>
       </c>
-      <c r="G2" s="16" t="n"/>
-      <c r="H2" s="16" t="n"/>
-      <c r="I2" s="16" t="n"/>
+      <c r="G2" s="16" t="inlineStr"/>
+      <c r="H2" s="17" t="n"/>
+      <c r="I2" s="17" t="n"/>
+      <c r="J2" s="17" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="14" t="inlineStr">
@@ -1209,9 +1231,10 @@
           <t>https://github.com/TechSckoolByVijay/75-day-career-upgrade/tree/main/week-00-setup</t>
         </is>
       </c>
-      <c r="G3" s="16" t="n"/>
-      <c r="H3" s="16" t="n"/>
-      <c r="I3" s="16" t="n"/>
+      <c r="G3" s="16" t="inlineStr"/>
+      <c r="H3" s="17" t="n"/>
+      <c r="I3" s="17" t="n"/>
+      <c r="J3" s="17" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="14" t="inlineStr">
@@ -1237,10 +1260,11 @@
           <t>Answer the 12 'Can I…?' questions in the Self-check tab (Start column). Be honest; nobody sees it but you.</t>
         </is>
       </c>
-      <c r="F4" s="17" t="inlineStr"/>
-      <c r="G4" s="16" t="n"/>
-      <c r="H4" s="16" t="n"/>
-      <c r="I4" s="16" t="n"/>
+      <c r="F4" s="16" t="inlineStr"/>
+      <c r="G4" s="16" t="inlineStr"/>
+      <c r="H4" s="17" t="n"/>
+      <c r="I4" s="17" t="n"/>
+      <c r="J4" s="17" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="14" t="inlineStr">
@@ -1266,29 +1290,30 @@
           <t>Write your one-sentence goal in the Start Here tab.</t>
         </is>
       </c>
-      <c r="F5" s="17" t="inlineStr"/>
-      <c r="G5" s="16" t="n"/>
-      <c r="H5" s="16" t="n"/>
-      <c r="I5" s="16" t="n"/>
+      <c r="F5" s="16" t="inlineStr"/>
+      <c r="G5" s="16" t="inlineStr"/>
+      <c r="H5" s="17" t="n"/>
+      <c r="I5" s="17" t="n"/>
+      <c r="J5" s="17" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="17" t="n">
+      <c r="A6" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="B6" s="17" t="n">
+      <c r="B6" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="C6" s="17" t="inlineStr">
-        <is>
-          <t>Learn</t>
-        </is>
-      </c>
-      <c r="D6" s="17" t="inlineStr">
+      <c r="C6" s="16" t="inlineStr">
+        <is>
+          <t>Learn</t>
+        </is>
+      </c>
+      <c r="D6" s="16" t="inlineStr">
         <is>
           <t>Foundations: Linux, Git, AI as your study partner</t>
         </is>
       </c>
-      <c r="E6" s="17" t="inlineStr">
+      <c r="E6" s="16" t="inlineStr">
         <is>
           <t>Terminal basics: pwd, ls, cd, mkdir, touch, cp, mv, rm. Practise until moving around feels normal.</t>
         </is>
@@ -1298,28 +1323,33 @@
           <t>https://ubuntu.com/tutorials/command-line-for-beginners</t>
         </is>
       </c>
-      <c r="G6" s="16" t="n"/>
-      <c r="H6" s="16" t="n"/>
-      <c r="I6" s="16" t="n"/>
+      <c r="G6" s="18" t="inlineStr">
+        <is>
+          <t>Not in our courses yet. The free resource is enough.</t>
+        </is>
+      </c>
+      <c r="H6" s="17" t="n"/>
+      <c r="I6" s="17" t="n"/>
+      <c r="J6" s="17" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="17" t="n">
+      <c r="A7" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="B7" s="17" t="n">
+      <c r="B7" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="C7" s="17" t="inlineStr">
-        <is>
-          <t>Learn</t>
-        </is>
-      </c>
-      <c r="D7" s="17" t="inlineStr">
+      <c r="C7" s="16" t="inlineStr">
+        <is>
+          <t>Learn</t>
+        </is>
+      </c>
+      <c r="D7" s="16" t="inlineStr">
         <is>
           <t>Foundations: Linux, Git, AI as your study partner</t>
         </is>
       </c>
-      <c r="E7" s="17" t="inlineStr">
+      <c r="E7" s="16" t="inlineStr">
         <is>
           <t>Working with text: cat, less, head, tail, grep, pipes ( | ) and redirection ( &gt; ).</t>
         </is>
@@ -1329,28 +1359,33 @@
           <t>https://linuxjourney.com/</t>
         </is>
       </c>
-      <c r="G7" s="16" t="n"/>
-      <c r="H7" s="16" t="n"/>
-      <c r="I7" s="16" t="n"/>
+      <c r="G7" s="18" t="inlineStr">
+        <is>
+          <t>Not in our courses yet. The free resource is enough.</t>
+        </is>
+      </c>
+      <c r="H7" s="17" t="n"/>
+      <c r="I7" s="17" t="n"/>
+      <c r="J7" s="17" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="17" t="n">
+      <c r="A8" s="16" t="n">
         <v>3</v>
       </c>
-      <c r="B8" s="17" t="n">
+      <c r="B8" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="C8" s="17" t="inlineStr">
-        <is>
-          <t>Learn</t>
-        </is>
-      </c>
-      <c r="D8" s="17" t="inlineStr">
+      <c r="C8" s="16" t="inlineStr">
+        <is>
+          <t>Learn</t>
+        </is>
+      </c>
+      <c r="D8" s="16" t="inlineStr">
         <is>
           <t>Foundations: Linux, Git, AI as your study partner</t>
         </is>
       </c>
-      <c r="E8" s="17" t="inlineStr">
+      <c r="E8" s="16" t="inlineStr">
         <is>
           <t>Permissions, processes and environment variables: chmod, ps, top, export, PATH.</t>
         </is>
@@ -1360,28 +1395,33 @@
           <t>https://linuxjourney.com/</t>
         </is>
       </c>
-      <c r="G8" s="16" t="n"/>
-      <c r="H8" s="16" t="n"/>
-      <c r="I8" s="16" t="n"/>
+      <c r="G8" s="18" t="inlineStr">
+        <is>
+          <t>Not in our courses yet. The free resource is enough.</t>
+        </is>
+      </c>
+      <c r="H8" s="17" t="n"/>
+      <c r="I8" s="17" t="n"/>
+      <c r="J8" s="17" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="17" t="n">
+      <c r="A9" s="16" t="n">
         <v>4</v>
       </c>
-      <c r="B9" s="17" t="n">
+      <c r="B9" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="C9" s="17" t="inlineStr">
-        <is>
-          <t>Learn</t>
-        </is>
-      </c>
-      <c r="D9" s="17" t="inlineStr">
+      <c r="C9" s="16" t="inlineStr">
+        <is>
+          <t>Learn</t>
+        </is>
+      </c>
+      <c r="D9" s="16" t="inlineStr">
         <is>
           <t>Foundations: Linux, Git, AI as your study partner</t>
         </is>
       </c>
-      <c r="E9" s="17" t="inlineStr">
+      <c r="E9" s="16" t="inlineStr">
         <is>
           <t>Git basics: init, add, commit, status, log. Create a GitHub repo and push your first commit.</t>
         </is>
@@ -1391,28 +1431,33 @@
           <t>https://docs.github.com/en/get-started/start-your-journey/hello-world</t>
         </is>
       </c>
-      <c r="G9" s="16" t="n"/>
-      <c r="H9" s="16" t="n"/>
-      <c r="I9" s="16" t="n"/>
+      <c r="G9" s="18" t="inlineStr">
+        <is>
+          <t>Not in our courses yet. The free resource is enough.</t>
+        </is>
+      </c>
+      <c r="H9" s="17" t="n"/>
+      <c r="I9" s="17" t="n"/>
+      <c r="J9" s="17" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="17" t="n">
+      <c r="A10" s="16" t="n">
         <v>5</v>
       </c>
-      <c r="B10" s="17" t="n">
+      <c r="B10" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="C10" s="17" t="inlineStr">
-        <is>
-          <t>Learn</t>
-        </is>
-      </c>
-      <c r="D10" s="17" t="inlineStr">
+      <c r="C10" s="16" t="inlineStr">
+        <is>
+          <t>Learn</t>
+        </is>
+      </c>
+      <c r="D10" s="16" t="inlineStr">
         <is>
           <t>Foundations: Linux, Git, AI as your study partner</t>
         </is>
       </c>
-      <c r="E10" s="17" t="inlineStr">
+      <c r="E10" s="16" t="inlineStr">
         <is>
           <t>AI as your study partner: give context + the exact error + your goal; check its answer; never paste passwords, keys or company data.</t>
         </is>
@@ -1422,9 +1467,14 @@
           <t>https://vijaysaini.com/blog-post.html?slug=ai-at-work-01-fit-in-dont-replace</t>
         </is>
       </c>
-      <c r="G10" s="16" t="n"/>
-      <c r="H10" s="16" t="n"/>
-      <c r="I10" s="16" t="n"/>
+      <c r="G10" s="15" t="inlineStr">
+        <is>
+          <t>ChatGPT for DevOps: "Leveraging ChatGPT - Ask to Explain the Code"</t>
+        </is>
+      </c>
+      <c r="H10" s="17" t="n"/>
+      <c r="I10" s="17" t="n"/>
+      <c r="J10" s="17" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="14" t="n">
@@ -1448,10 +1498,15 @@
           <t>Write a small shell script that shows disk usage and the 5 largest files in a folder. Push it to GitHub. Ask AI to review it and explain one improvement.</t>
         </is>
       </c>
-      <c r="F11" s="17" t="inlineStr"/>
-      <c r="G11" s="16" t="n"/>
-      <c r="H11" s="16" t="n"/>
-      <c r="I11" s="16" t="n"/>
+      <c r="F11" s="16" t="inlineStr"/>
+      <c r="G11" s="15" t="inlineStr">
+        <is>
+          <t>ChatGPT for DevOps: "Harnessing the Power of ChatGPT - Coding with ChatGPT"</t>
+        </is>
+      </c>
+      <c r="H11" s="17" t="n"/>
+      <c r="I11" s="17" t="n"/>
+      <c r="J11" s="17" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="14" t="n">
@@ -1475,29 +1530,30 @@
           <t>Finish anything left from the week. Write your weekly reflection in the Weekly tab.</t>
         </is>
       </c>
-      <c r="F12" s="17" t="inlineStr"/>
-      <c r="G12" s="16" t="n"/>
-      <c r="H12" s="16" t="n"/>
-      <c r="I12" s="16" t="n"/>
+      <c r="F12" s="16" t="inlineStr"/>
+      <c r="G12" s="16" t="inlineStr"/>
+      <c r="H12" s="17" t="n"/>
+      <c r="I12" s="17" t="n"/>
+      <c r="J12" s="17" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="17" t="n">
+      <c r="A13" s="16" t="n">
         <v>8</v>
       </c>
-      <c r="B13" s="17" t="n">
+      <c r="B13" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="C13" s="17" t="inlineStr">
-        <is>
-          <t>Learn</t>
-        </is>
-      </c>
-      <c r="D13" s="17" t="inlineStr">
+      <c r="C13" s="16" t="inlineStr">
+        <is>
+          <t>Learn</t>
+        </is>
+      </c>
+      <c r="D13" s="16" t="inlineStr">
         <is>
           <t>Docker</t>
         </is>
       </c>
-      <c r="E13" s="17" t="inlineStr">
+      <c r="E13" s="16" t="inlineStr">
         <is>
           <t>Containers vs virtual machines. Run nginx: docker run -p 8080:80 nginx, then open localhost:8080.</t>
         </is>
@@ -1507,28 +1563,33 @@
           <t>https://docs.docker.com/get-started/</t>
         </is>
       </c>
-      <c r="G13" s="16" t="n"/>
-      <c r="H13" s="16" t="n"/>
-      <c r="I13" s="16" t="n"/>
+      <c r="G13" s="18" t="inlineStr">
+        <is>
+          <t>Not in our courses yet. The free resource is enough.</t>
+        </is>
+      </c>
+      <c r="H13" s="17" t="n"/>
+      <c r="I13" s="17" t="n"/>
+      <c r="J13" s="17" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="17" t="n">
+      <c r="A14" s="16" t="n">
         <v>9</v>
       </c>
-      <c r="B14" s="17" t="n">
+      <c r="B14" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="C14" s="17" t="inlineStr">
-        <is>
-          <t>Learn</t>
-        </is>
-      </c>
-      <c r="D14" s="17" t="inlineStr">
+      <c r="C14" s="16" t="inlineStr">
+        <is>
+          <t>Learn</t>
+        </is>
+      </c>
+      <c r="D14" s="16" t="inlineStr">
         <is>
           <t>Docker</t>
         </is>
       </c>
-      <c r="E14" s="17" t="inlineStr">
+      <c r="E14" s="16" t="inlineStr">
         <is>
           <t>Images and containers: docker ps, images, logs, exec, stop, rm. Look inside a running container.</t>
         </is>
@@ -1538,28 +1599,33 @@
           <t>https://docs.docker.com/get-started/</t>
         </is>
       </c>
-      <c r="G14" s="16" t="n"/>
-      <c r="H14" s="16" t="n"/>
-      <c r="I14" s="16" t="n"/>
+      <c r="G14" s="18" t="inlineStr">
+        <is>
+          <t>Not in our courses yet. The free resource is enough.</t>
+        </is>
+      </c>
+      <c r="H14" s="17" t="n"/>
+      <c r="I14" s="17" t="n"/>
+      <c r="J14" s="17" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="17" t="n">
+      <c r="A15" s="16" t="n">
         <v>10</v>
       </c>
-      <c r="B15" s="17" t="n">
+      <c r="B15" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="C15" s="17" t="inlineStr">
-        <is>
-          <t>Learn</t>
-        </is>
-      </c>
-      <c r="D15" s="17" t="inlineStr">
+      <c r="C15" s="16" t="inlineStr">
+        <is>
+          <t>Learn</t>
+        </is>
+      </c>
+      <c r="D15" s="16" t="inlineStr">
         <is>
           <t>Docker</t>
         </is>
       </c>
-      <c r="E15" s="17" t="inlineStr">
+      <c r="E15" s="16" t="inlineStr">
         <is>
           <t>Write a Dockerfile for a tiny Python app (or read the Notes app's Dockerfile line by line), build it and run it.</t>
         </is>
@@ -1569,28 +1635,33 @@
           <t>https://docs.docker.com/get-started/workshop/</t>
         </is>
       </c>
-      <c r="G15" s="16" t="n"/>
-      <c r="H15" s="16" t="n"/>
-      <c r="I15" s="16" t="n"/>
+      <c r="G15" s="15" t="inlineStr">
+        <is>
+          <t>ChatGPT for DevOps: "Use ChatGPT for Generating Dockerfile"</t>
+        </is>
+      </c>
+      <c r="H15" s="17" t="n"/>
+      <c r="I15" s="17" t="n"/>
+      <c r="J15" s="17" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="17" t="n">
+      <c r="A16" s="16" t="n">
         <v>11</v>
       </c>
-      <c r="B16" s="17" t="n">
+      <c r="B16" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="C16" s="17" t="inlineStr">
-        <is>
-          <t>Learn</t>
-        </is>
-      </c>
-      <c r="D16" s="17" t="inlineStr">
+      <c r="C16" s="16" t="inlineStr">
+        <is>
+          <t>Learn</t>
+        </is>
+      </c>
+      <c r="D16" s="16" t="inlineStr">
         <is>
           <t>Docker</t>
         </is>
       </c>
-      <c r="E16" s="17" t="inlineStr">
+      <c r="E16" s="16" t="inlineStr">
         <is>
           <t>Environment variables, volumes and .dockerignore: keep secrets OUT of the image.</t>
         </is>
@@ -1600,28 +1671,33 @@
           <t>https://docs.docker.com/build/concepts/context/#dockerignore-files</t>
         </is>
       </c>
-      <c r="G16" s="16" t="n"/>
-      <c r="H16" s="16" t="n"/>
-      <c r="I16" s="16" t="n"/>
+      <c r="G16" s="18" t="inlineStr">
+        <is>
+          <t>Not in our courses yet. The free resource is enough.</t>
+        </is>
+      </c>
+      <c r="H16" s="17" t="n"/>
+      <c r="I16" s="17" t="n"/>
+      <c r="J16" s="17" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="17" t="n">
+      <c r="A17" s="16" t="n">
         <v>12</v>
       </c>
-      <c r="B17" s="17" t="n">
+      <c r="B17" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="C17" s="17" t="inlineStr">
-        <is>
-          <t>Learn</t>
-        </is>
-      </c>
-      <c r="D17" s="17" t="inlineStr">
+      <c r="C17" s="16" t="inlineStr">
+        <is>
+          <t>Learn</t>
+        </is>
+      </c>
+      <c r="D17" s="16" t="inlineStr">
         <is>
           <t>Docker</t>
         </is>
       </c>
-      <c r="E17" s="17" t="inlineStr">
+      <c r="E17" s="16" t="inlineStr">
         <is>
           <t>Run 2 containers together: the Notes app + Redis, first with docker network, then with Docker Compose.</t>
         </is>
@@ -1631,9 +1707,14 @@
           <t>https://docs.docker.com/compose/gettingstarted/</t>
         </is>
       </c>
-      <c r="G17" s="16" t="n"/>
-      <c r="H17" s="16" t="n"/>
-      <c r="I17" s="16" t="n"/>
+      <c r="G17" s="18" t="inlineStr">
+        <is>
+          <t>Not in our courses yet. The free resource is enough.</t>
+        </is>
+      </c>
+      <c r="H17" s="17" t="n"/>
+      <c r="I17" s="17" t="n"/>
+      <c r="J17" s="17" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="14" t="n">
@@ -1662,9 +1743,14 @@
           <t>https://github.com/TechSckoolByVijay/75-day-career-upgrade/tree/main/apps/notes-app</t>
         </is>
       </c>
-      <c r="G18" s="16" t="n"/>
-      <c r="H18" s="16" t="n"/>
-      <c r="I18" s="16" t="n"/>
+      <c r="G18" s="15" t="inlineStr">
+        <is>
+          <t>ChatGPT for DevOps: "Use ChatGPT for Generating Dockerfile (use it to review yours)"</t>
+        </is>
+      </c>
+      <c r="H18" s="17" t="n"/>
+      <c r="I18" s="17" t="n"/>
+      <c r="J18" s="17" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="14" t="n">
@@ -1688,29 +1774,30 @@
           <t>Finish the week. Weekly reflection.</t>
         </is>
       </c>
-      <c r="F19" s="17" t="inlineStr"/>
-      <c r="G19" s="16" t="n"/>
-      <c r="H19" s="16" t="n"/>
-      <c r="I19" s="16" t="n"/>
+      <c r="F19" s="16" t="inlineStr"/>
+      <c r="G19" s="16" t="inlineStr"/>
+      <c r="H19" s="17" t="n"/>
+      <c r="I19" s="17" t="n"/>
+      <c r="J19" s="17" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="17" t="n">
+      <c r="A20" s="16" t="n">
         <v>15</v>
       </c>
-      <c r="B20" s="17" t="n">
+      <c r="B20" s="16" t="n">
         <v>3</v>
       </c>
-      <c r="C20" s="17" t="inlineStr">
-        <is>
-          <t>Learn</t>
-        </is>
-      </c>
-      <c r="D20" s="17" t="inlineStr">
+      <c r="C20" s="16" t="inlineStr">
+        <is>
+          <t>Learn</t>
+        </is>
+      </c>
+      <c r="D20" s="16" t="inlineStr">
         <is>
           <t>Kubernetes I</t>
         </is>
       </c>
-      <c r="E20" s="17" t="inlineStr">
+      <c r="E20" s="16" t="inlineStr">
         <is>
           <t>Why Kubernetes exists. Create a kind cluster; kubectl get nodes; kubectl explain pod.</t>
         </is>
@@ -1720,28 +1807,33 @@
           <t>https://kubernetes.io/docs/tutorials/kubernetes-basics/</t>
         </is>
       </c>
-      <c r="G20" s="16" t="n"/>
-      <c r="H20" s="16" t="n"/>
-      <c r="I20" s="16" t="n"/>
+      <c r="G20" s="15" t="inlineStr">
+        <is>
+          <t>Hands On Kubernetes: "Introduction to Kubernetes project &amp; basic commands overview"</t>
+        </is>
+      </c>
+      <c r="H20" s="17" t="n"/>
+      <c r="I20" s="17" t="n"/>
+      <c r="J20" s="17" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="17" t="n">
+      <c r="A21" s="16" t="n">
         <v>16</v>
       </c>
-      <c r="B21" s="17" t="n">
+      <c r="B21" s="16" t="n">
         <v>3</v>
       </c>
-      <c r="C21" s="17" t="inlineStr">
-        <is>
-          <t>Learn</t>
-        </is>
-      </c>
-      <c r="D21" s="17" t="inlineStr">
+      <c r="C21" s="16" t="inlineStr">
+        <is>
+          <t>Learn</t>
+        </is>
+      </c>
+      <c r="D21" s="16" t="inlineStr">
         <is>
           <t>Kubernetes I</t>
         </is>
       </c>
-      <c r="E21" s="17" t="inlineStr">
+      <c r="E21" s="16" t="inlineStr">
         <is>
           <t>Pods: run one, describe it, read its logs, delete it. Read a pod YAML line by line.</t>
         </is>
@@ -1751,28 +1843,33 @@
           <t>https://kubernetes.io/docs/concepts/workloads/pods/</t>
         </is>
       </c>
-      <c r="G21" s="16" t="n"/>
-      <c r="H21" s="16" t="n"/>
-      <c r="I21" s="16" t="n"/>
+      <c r="G21" s="15" t="inlineStr">
+        <is>
+          <t>Hands On Kubernetes: "Introduction to Kubernetes project &amp; basic commands overview"</t>
+        </is>
+      </c>
+      <c r="H21" s="17" t="n"/>
+      <c r="I21" s="17" t="n"/>
+      <c r="J21" s="17" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="17" t="n">
+      <c r="A22" s="16" t="n">
         <v>17</v>
       </c>
-      <c r="B22" s="17" t="n">
+      <c r="B22" s="16" t="n">
         <v>3</v>
       </c>
-      <c r="C22" s="17" t="inlineStr">
-        <is>
-          <t>Learn</t>
-        </is>
-      </c>
-      <c r="D22" s="17" t="inlineStr">
+      <c r="C22" s="16" t="inlineStr">
+        <is>
+          <t>Learn</t>
+        </is>
+      </c>
+      <c r="D22" s="16" t="inlineStr">
         <is>
           <t>Kubernetes I</t>
         </is>
       </c>
-      <c r="E22" s="17" t="inlineStr">
+      <c r="E22" s="16" t="inlineStr">
         <is>
           <t>Deployments: create, scale, roll out a new version, roll back.</t>
         </is>
@@ -1782,28 +1879,33 @@
           <t>https://kubernetes.io/docs/concepts/workloads/controllers/deployment/</t>
         </is>
       </c>
-      <c r="G22" s="16" t="n"/>
-      <c r="H22" s="16" t="n"/>
-      <c r="I22" s="16" t="n"/>
+      <c r="G22" s="15" t="inlineStr">
+        <is>
+          <t>Hands On Kubernetes: "Kubernetes Deployments: Streamlining Application Deployment"</t>
+        </is>
+      </c>
+      <c r="H22" s="17" t="n"/>
+      <c r="I22" s="17" t="n"/>
+      <c r="J22" s="17" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="17" t="n">
+      <c r="A23" s="16" t="n">
         <v>18</v>
       </c>
-      <c r="B23" s="17" t="n">
+      <c r="B23" s="16" t="n">
         <v>3</v>
       </c>
-      <c r="C23" s="17" t="inlineStr">
-        <is>
-          <t>Learn</t>
-        </is>
-      </c>
-      <c r="D23" s="17" t="inlineStr">
+      <c r="C23" s="16" t="inlineStr">
+        <is>
+          <t>Learn</t>
+        </is>
+      </c>
+      <c r="D23" s="16" t="inlineStr">
         <is>
           <t>Kubernetes I</t>
         </is>
       </c>
-      <c r="E23" s="17" t="inlineStr">
+      <c r="E23" s="16" t="inlineStr">
         <is>
           <t>Services, labels and selectors: ClusterIP vs NodePort; kubectl port-forward.</t>
         </is>
@@ -1813,28 +1915,33 @@
           <t>https://kubernetes.io/docs/concepts/services-networking/service/</t>
         </is>
       </c>
-      <c r="G23" s="16" t="n"/>
-      <c r="H23" s="16" t="n"/>
-      <c r="I23" s="16" t="n"/>
+      <c r="G23" s="15" t="inlineStr">
+        <is>
+          <t>Hands On Kubernetes: "Project Lab: Scaling a Multi-Tier Web Application"</t>
+        </is>
+      </c>
+      <c r="H23" s="17" t="n"/>
+      <c r="I23" s="17" t="n"/>
+      <c r="J23" s="17" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="17" t="n">
+      <c r="A24" s="16" t="n">
         <v>19</v>
       </c>
-      <c r="B24" s="17" t="n">
+      <c r="B24" s="16" t="n">
         <v>3</v>
       </c>
-      <c r="C24" s="17" t="inlineStr">
-        <is>
-          <t>Learn</t>
-        </is>
-      </c>
-      <c r="D24" s="17" t="inlineStr">
+      <c r="C24" s="16" t="inlineStr">
+        <is>
+          <t>Learn</t>
+        </is>
+      </c>
+      <c r="D24" s="16" t="inlineStr">
         <is>
           <t>Kubernetes I</t>
         </is>
       </c>
-      <c r="E24" s="17" t="inlineStr">
+      <c r="E24" s="16" t="inlineStr">
         <is>
           <t>Namespaces and kubectl productivity: -o wide, -o yaml, get events, describe.</t>
         </is>
@@ -1844,9 +1951,14 @@
           <t>https://kubernetes.io/docs/reference/kubectl/quick-reference/</t>
         </is>
       </c>
-      <c r="G24" s="16" t="n"/>
-      <c r="H24" s="16" t="n"/>
-      <c r="I24" s="16" t="n"/>
+      <c r="G24" s="15" t="inlineStr">
+        <is>
+          <t>Hands On Kubernetes: "Introduction to Kubernetes project &amp; basic commands overview"</t>
+        </is>
+      </c>
+      <c r="H24" s="17" t="n"/>
+      <c r="I24" s="17" t="n"/>
+      <c r="J24" s="17" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="14" t="n">
@@ -1875,9 +1987,14 @@
           <t>https://github.com/TechSckoolByVijay/75-day-career-upgrade/tree/main/week-03-kubernetes-1</t>
         </is>
       </c>
-      <c r="G25" s="16" t="n"/>
-      <c r="H25" s="16" t="n"/>
-      <c r="I25" s="16" t="n"/>
+      <c r="G25" s="15" t="inlineStr">
+        <is>
+          <t>k8s Production Readiness: "k8s live troubleshooting, parts 1-4"</t>
+        </is>
+      </c>
+      <c r="H25" s="17" t="n"/>
+      <c r="I25" s="17" t="n"/>
+      <c r="J25" s="17" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="14" t="n">
@@ -1901,29 +2018,30 @@
           <t>Finish the week. Weekly reflection.</t>
         </is>
       </c>
-      <c r="F26" s="17" t="inlineStr"/>
-      <c r="G26" s="16" t="n"/>
-      <c r="H26" s="16" t="n"/>
-      <c r="I26" s="16" t="n"/>
+      <c r="F26" s="16" t="inlineStr"/>
+      <c r="G26" s="16" t="inlineStr"/>
+      <c r="H26" s="17" t="n"/>
+      <c r="I26" s="17" t="n"/>
+      <c r="J26" s="17" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="17" t="n">
+      <c r="A27" s="16" t="n">
         <v>22</v>
       </c>
-      <c r="B27" s="17" t="n">
+      <c r="B27" s="16" t="n">
         <v>4</v>
       </c>
-      <c r="C27" s="17" t="inlineStr">
-        <is>
-          <t>Learn</t>
-        </is>
-      </c>
-      <c r="D27" s="17" t="inlineStr">
+      <c r="C27" s="16" t="inlineStr">
+        <is>
+          <t>Learn</t>
+        </is>
+      </c>
+      <c r="D27" s="16" t="inlineStr">
         <is>
           <t>Kubernetes II: production basics</t>
         </is>
       </c>
-      <c r="E27" s="17" t="inlineStr">
+      <c r="E27" s="16" t="inlineStr">
         <is>
           <t>Opens when Week 4 starts: see the Week 4 lesson. (Kubernetes II: production basics)</t>
         </is>
@@ -1933,28 +2051,33 @@
           <t>https://github.com/TechSckoolByVijay/75-day-career-upgrade/tree/main/week-04-kubernetes-2</t>
         </is>
       </c>
-      <c r="G27" s="16" t="n"/>
-      <c r="H27" s="16" t="n"/>
-      <c r="I27" s="16" t="n"/>
+      <c r="G27" s="15" t="inlineStr">
+        <is>
+          <t>Hands On Kubernetes: "Resource Requests &amp; Limits; ConfigMaps and Secrets; Persistent Volumes" · k8s Production Readiness: "Production Incident Response &amp; Live Troubleshooting"</t>
+        </is>
+      </c>
+      <c r="H27" s="17" t="n"/>
+      <c r="I27" s="17" t="n"/>
+      <c r="J27" s="17" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="17" t="n">
+      <c r="A28" s="16" t="n">
         <v>23</v>
       </c>
-      <c r="B28" s="17" t="n">
+      <c r="B28" s="16" t="n">
         <v>4</v>
       </c>
-      <c r="C28" s="17" t="inlineStr">
-        <is>
-          <t>Learn</t>
-        </is>
-      </c>
-      <c r="D28" s="17" t="inlineStr">
+      <c r="C28" s="16" t="inlineStr">
+        <is>
+          <t>Learn</t>
+        </is>
+      </c>
+      <c r="D28" s="16" t="inlineStr">
         <is>
           <t>Kubernetes II: production basics</t>
         </is>
       </c>
-      <c r="E28" s="17" t="inlineStr">
+      <c r="E28" s="16" t="inlineStr">
         <is>
           <t>Opens when Week 4 starts: see the Week 4 lesson. (Kubernetes II: production basics)</t>
         </is>
@@ -1964,28 +2087,33 @@
           <t>https://github.com/TechSckoolByVijay/75-day-career-upgrade/tree/main/week-04-kubernetes-2</t>
         </is>
       </c>
-      <c r="G28" s="16" t="n"/>
-      <c r="H28" s="16" t="n"/>
-      <c r="I28" s="16" t="n"/>
+      <c r="G28" s="15" t="inlineStr">
+        <is>
+          <t>Hands On Kubernetes: "Resource Requests &amp; Limits; ConfigMaps and Secrets; Persistent Volumes" · k8s Production Readiness: "Production Incident Response &amp; Live Troubleshooting"</t>
+        </is>
+      </c>
+      <c r="H28" s="17" t="n"/>
+      <c r="I28" s="17" t="n"/>
+      <c r="J28" s="17" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="17" t="n">
+      <c r="A29" s="16" t="n">
         <v>24</v>
       </c>
-      <c r="B29" s="17" t="n">
+      <c r="B29" s="16" t="n">
         <v>4</v>
       </c>
-      <c r="C29" s="17" t="inlineStr">
-        <is>
-          <t>Learn</t>
-        </is>
-      </c>
-      <c r="D29" s="17" t="inlineStr">
+      <c r="C29" s="16" t="inlineStr">
+        <is>
+          <t>Learn</t>
+        </is>
+      </c>
+      <c r="D29" s="16" t="inlineStr">
         <is>
           <t>Kubernetes II: production basics</t>
         </is>
       </c>
-      <c r="E29" s="17" t="inlineStr">
+      <c r="E29" s="16" t="inlineStr">
         <is>
           <t>Opens when Week 4 starts: see the Week 4 lesson. (Kubernetes II: production basics)</t>
         </is>
@@ -1995,28 +2123,33 @@
           <t>https://github.com/TechSckoolByVijay/75-day-career-upgrade/tree/main/week-04-kubernetes-2</t>
         </is>
       </c>
-      <c r="G29" s="16" t="n"/>
-      <c r="H29" s="16" t="n"/>
-      <c r="I29" s="16" t="n"/>
+      <c r="G29" s="15" t="inlineStr">
+        <is>
+          <t>Hands On Kubernetes: "Resource Requests &amp; Limits; ConfigMaps and Secrets; Persistent Volumes" · k8s Production Readiness: "Production Incident Response &amp; Live Troubleshooting"</t>
+        </is>
+      </c>
+      <c r="H29" s="17" t="n"/>
+      <c r="I29" s="17" t="n"/>
+      <c r="J29" s="17" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="17" t="n">
+      <c r="A30" s="16" t="n">
         <v>25</v>
       </c>
-      <c r="B30" s="17" t="n">
+      <c r="B30" s="16" t="n">
         <v>4</v>
       </c>
-      <c r="C30" s="17" t="inlineStr">
-        <is>
-          <t>Learn</t>
-        </is>
-      </c>
-      <c r="D30" s="17" t="inlineStr">
+      <c r="C30" s="16" t="inlineStr">
+        <is>
+          <t>Learn</t>
+        </is>
+      </c>
+      <c r="D30" s="16" t="inlineStr">
         <is>
           <t>Kubernetes II: production basics</t>
         </is>
       </c>
-      <c r="E30" s="17" t="inlineStr">
+      <c r="E30" s="16" t="inlineStr">
         <is>
           <t>Opens when Week 4 starts: see the Week 4 lesson. (Kubernetes II: production basics)</t>
         </is>
@@ -2026,28 +2159,33 @@
           <t>https://github.com/TechSckoolByVijay/75-day-career-upgrade/tree/main/week-04-kubernetes-2</t>
         </is>
       </c>
-      <c r="G30" s="16" t="n"/>
-      <c r="H30" s="16" t="n"/>
-      <c r="I30" s="16" t="n"/>
+      <c r="G30" s="15" t="inlineStr">
+        <is>
+          <t>Hands On Kubernetes: "Resource Requests &amp; Limits; ConfigMaps and Secrets; Persistent Volumes" · k8s Production Readiness: "Production Incident Response &amp; Live Troubleshooting"</t>
+        </is>
+      </c>
+      <c r="H30" s="17" t="n"/>
+      <c r="I30" s="17" t="n"/>
+      <c r="J30" s="17" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="17" t="n">
+      <c r="A31" s="16" t="n">
         <v>26</v>
       </c>
-      <c r="B31" s="17" t="n">
+      <c r="B31" s="16" t="n">
         <v>4</v>
       </c>
-      <c r="C31" s="17" t="inlineStr">
-        <is>
-          <t>Learn</t>
-        </is>
-      </c>
-      <c r="D31" s="17" t="inlineStr">
+      <c r="C31" s="16" t="inlineStr">
+        <is>
+          <t>Learn</t>
+        </is>
+      </c>
+      <c r="D31" s="16" t="inlineStr">
         <is>
           <t>Kubernetes II: production basics</t>
         </is>
       </c>
-      <c r="E31" s="17" t="inlineStr">
+      <c r="E31" s="16" t="inlineStr">
         <is>
           <t>Opens when Week 4 starts: see the Week 4 lesson. (Kubernetes II: production basics)</t>
         </is>
@@ -2057,9 +2195,14 @@
           <t>https://github.com/TechSckoolByVijay/75-day-career-upgrade/tree/main/week-04-kubernetes-2</t>
         </is>
       </c>
-      <c r="G31" s="16" t="n"/>
-      <c r="H31" s="16" t="n"/>
-      <c r="I31" s="16" t="n"/>
+      <c r="G31" s="15" t="inlineStr">
+        <is>
+          <t>Hands On Kubernetes: "Resource Requests &amp; Limits; ConfigMaps and Secrets; Persistent Volumes" · k8s Production Readiness: "Production Incident Response &amp; Live Troubleshooting"</t>
+        </is>
+      </c>
+      <c r="H31" s="17" t="n"/>
+      <c r="I31" s="17" t="n"/>
+      <c r="J31" s="17" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="14" t="n">
@@ -2088,9 +2231,14 @@
           <t>https://github.com/TechSckoolByVijay/75-day-career-upgrade/tree/main/week-04-kubernetes-2</t>
         </is>
       </c>
-      <c r="G32" s="16" t="n"/>
-      <c r="H32" s="16" t="n"/>
-      <c r="I32" s="16" t="n"/>
+      <c r="G32" s="15" t="inlineStr">
+        <is>
+          <t>Hands On Kubernetes: "Resource Requests &amp; Limits; ConfigMaps and Secrets; Persistent Volumes" · k8s Production Readiness: "Production Incident Response &amp; Live Troubleshooting"</t>
+        </is>
+      </c>
+      <c r="H32" s="17" t="n"/>
+      <c r="I32" s="17" t="n"/>
+      <c r="J32" s="17" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="14" t="n">
@@ -2119,28 +2267,33 @@
           <t>https://github.com/TechSckoolByVijay/75-day-career-upgrade/tree/main/week-04-kubernetes-2</t>
         </is>
       </c>
-      <c r="G33" s="16" t="n"/>
-      <c r="H33" s="16" t="n"/>
-      <c r="I33" s="16" t="n"/>
+      <c r="G33" s="15" t="inlineStr">
+        <is>
+          <t>Hands On Kubernetes: "Resource Requests &amp; Limits; ConfigMaps and Secrets; Persistent Volumes" · k8s Production Readiness: "Production Incident Response &amp; Live Troubleshooting"</t>
+        </is>
+      </c>
+      <c r="H33" s="17" t="n"/>
+      <c r="I33" s="17" t="n"/>
+      <c r="J33" s="17" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" s="17" t="n">
+      <c r="A34" s="16" t="n">
         <v>29</v>
       </c>
-      <c r="B34" s="17" t="n">
+      <c r="B34" s="16" t="n">
         <v>5</v>
       </c>
-      <c r="C34" s="17" t="inlineStr">
-        <is>
-          <t>Learn</t>
-        </is>
-      </c>
-      <c r="D34" s="17" t="inlineStr">
+      <c r="C34" s="16" t="inlineStr">
+        <is>
+          <t>Learn</t>
+        </is>
+      </c>
+      <c r="D34" s="16" t="inlineStr">
         <is>
           <t>Checkpoint 1: projects + self-check</t>
         </is>
       </c>
-      <c r="E34" s="17" t="inlineStr">
+      <c r="E34" s="16" t="inlineStr">
         <is>
           <t>Opens when Week 5 starts: see the Week 5 lesson. (Checkpoint 1: projects + self-check)</t>
         </is>
@@ -2150,28 +2303,33 @@
           <t>https://github.com/TechSckoolByVijay/75-day-career-upgrade/tree/main/week-05-checkpoint-1</t>
         </is>
       </c>
-      <c r="G34" s="16" t="n"/>
-      <c r="H34" s="16" t="n"/>
-      <c r="I34" s="16" t="n"/>
+      <c r="G34" s="15" t="inlineStr">
+        <is>
+          <t>Hands On Kubernetes: "Project Lab: Scaling a Multi-Tier Web Application"</t>
+        </is>
+      </c>
+      <c r="H34" s="17" t="n"/>
+      <c r="I34" s="17" t="n"/>
+      <c r="J34" s="17" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="17" t="n">
+      <c r="A35" s="16" t="n">
         <v>30</v>
       </c>
-      <c r="B35" s="17" t="n">
+      <c r="B35" s="16" t="n">
         <v>5</v>
       </c>
-      <c r="C35" s="17" t="inlineStr">
-        <is>
-          <t>Learn</t>
-        </is>
-      </c>
-      <c r="D35" s="17" t="inlineStr">
+      <c r="C35" s="16" t="inlineStr">
+        <is>
+          <t>Learn</t>
+        </is>
+      </c>
+      <c r="D35" s="16" t="inlineStr">
         <is>
           <t>Checkpoint 1: projects + self-check</t>
         </is>
       </c>
-      <c r="E35" s="17" t="inlineStr">
+      <c r="E35" s="16" t="inlineStr">
         <is>
           <t>Opens when Week 5 starts: see the Week 5 lesson. (Checkpoint 1: projects + self-check)</t>
         </is>
@@ -2181,28 +2339,33 @@
           <t>https://github.com/TechSckoolByVijay/75-day-career-upgrade/tree/main/week-05-checkpoint-1</t>
         </is>
       </c>
-      <c r="G35" s="16" t="n"/>
-      <c r="H35" s="16" t="n"/>
-      <c r="I35" s="16" t="n"/>
+      <c r="G35" s="15" t="inlineStr">
+        <is>
+          <t>Hands On Kubernetes: "Project Lab: Scaling a Multi-Tier Web Application"</t>
+        </is>
+      </c>
+      <c r="H35" s="17" t="n"/>
+      <c r="I35" s="17" t="n"/>
+      <c r="J35" s="17" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="17" t="n">
+      <c r="A36" s="16" t="n">
         <v>31</v>
       </c>
-      <c r="B36" s="17" t="n">
+      <c r="B36" s="16" t="n">
         <v>5</v>
       </c>
-      <c r="C36" s="17" t="inlineStr">
-        <is>
-          <t>Learn</t>
-        </is>
-      </c>
-      <c r="D36" s="17" t="inlineStr">
+      <c r="C36" s="16" t="inlineStr">
+        <is>
+          <t>Learn</t>
+        </is>
+      </c>
+      <c r="D36" s="16" t="inlineStr">
         <is>
           <t>Checkpoint 1: projects + self-check</t>
         </is>
       </c>
-      <c r="E36" s="17" t="inlineStr">
+      <c r="E36" s="16" t="inlineStr">
         <is>
           <t>Opens when Week 5 starts: see the Week 5 lesson. (Checkpoint 1: projects + self-check)</t>
         </is>
@@ -2212,28 +2375,33 @@
           <t>https://github.com/TechSckoolByVijay/75-day-career-upgrade/tree/main/week-05-checkpoint-1</t>
         </is>
       </c>
-      <c r="G36" s="16" t="n"/>
-      <c r="H36" s="16" t="n"/>
-      <c r="I36" s="16" t="n"/>
+      <c r="G36" s="15" t="inlineStr">
+        <is>
+          <t>Hands On Kubernetes: "Project Lab: Scaling a Multi-Tier Web Application"</t>
+        </is>
+      </c>
+      <c r="H36" s="17" t="n"/>
+      <c r="I36" s="17" t="n"/>
+      <c r="J36" s="17" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="17" t="n">
+      <c r="A37" s="16" t="n">
         <v>32</v>
       </c>
-      <c r="B37" s="17" t="n">
+      <c r="B37" s="16" t="n">
         <v>5</v>
       </c>
-      <c r="C37" s="17" t="inlineStr">
-        <is>
-          <t>Learn</t>
-        </is>
-      </c>
-      <c r="D37" s="17" t="inlineStr">
+      <c r="C37" s="16" t="inlineStr">
+        <is>
+          <t>Learn</t>
+        </is>
+      </c>
+      <c r="D37" s="16" t="inlineStr">
         <is>
           <t>Checkpoint 1: projects + self-check</t>
         </is>
       </c>
-      <c r="E37" s="17" t="inlineStr">
+      <c r="E37" s="16" t="inlineStr">
         <is>
           <t>Opens when Week 5 starts: see the Week 5 lesson. (Checkpoint 1: projects + self-check)</t>
         </is>
@@ -2243,28 +2411,33 @@
           <t>https://github.com/TechSckoolByVijay/75-day-career-upgrade/tree/main/week-05-checkpoint-1</t>
         </is>
       </c>
-      <c r="G37" s="16" t="n"/>
-      <c r="H37" s="16" t="n"/>
-      <c r="I37" s="16" t="n"/>
+      <c r="G37" s="15" t="inlineStr">
+        <is>
+          <t>Hands On Kubernetes: "Project Lab: Scaling a Multi-Tier Web Application"</t>
+        </is>
+      </c>
+      <c r="H37" s="17" t="n"/>
+      <c r="I37" s="17" t="n"/>
+      <c r="J37" s="17" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" s="17" t="n">
+      <c r="A38" s="16" t="n">
         <v>33</v>
       </c>
-      <c r="B38" s="17" t="n">
+      <c r="B38" s="16" t="n">
         <v>5</v>
       </c>
-      <c r="C38" s="17" t="inlineStr">
-        <is>
-          <t>Learn</t>
-        </is>
-      </c>
-      <c r="D38" s="17" t="inlineStr">
+      <c r="C38" s="16" t="inlineStr">
+        <is>
+          <t>Learn</t>
+        </is>
+      </c>
+      <c r="D38" s="16" t="inlineStr">
         <is>
           <t>Checkpoint 1: projects + self-check</t>
         </is>
       </c>
-      <c r="E38" s="17" t="inlineStr">
+      <c r="E38" s="16" t="inlineStr">
         <is>
           <t>Opens when Week 5 starts: see the Week 5 lesson. (Checkpoint 1: projects + self-check)</t>
         </is>
@@ -2274,9 +2447,14 @@
           <t>https://github.com/TechSckoolByVijay/75-day-career-upgrade/tree/main/week-05-checkpoint-1</t>
         </is>
       </c>
-      <c r="G38" s="16" t="n"/>
-      <c r="H38" s="16" t="n"/>
-      <c r="I38" s="16" t="n"/>
+      <c r="G38" s="15" t="inlineStr">
+        <is>
+          <t>Hands On Kubernetes: "Project Lab: Scaling a Multi-Tier Web Application"</t>
+        </is>
+      </c>
+      <c r="H38" s="17" t="n"/>
+      <c r="I38" s="17" t="n"/>
+      <c r="J38" s="17" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="14" t="n">
@@ -2305,9 +2483,14 @@
           <t>https://github.com/TechSckoolByVijay/75-day-career-upgrade/tree/main/week-05-checkpoint-1</t>
         </is>
       </c>
-      <c r="G39" s="16" t="n"/>
-      <c r="H39" s="16" t="n"/>
-      <c r="I39" s="16" t="n"/>
+      <c r="G39" s="15" t="inlineStr">
+        <is>
+          <t>Hands On Kubernetes: "Project Lab: Scaling a Multi-Tier Web Application"</t>
+        </is>
+      </c>
+      <c r="H39" s="17" t="n"/>
+      <c r="I39" s="17" t="n"/>
+      <c r="J39" s="17" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="14" t="n">
@@ -2336,28 +2519,33 @@
           <t>https://github.com/TechSckoolByVijay/75-day-career-upgrade/tree/main/week-05-checkpoint-1</t>
         </is>
       </c>
-      <c r="G40" s="16" t="n"/>
-      <c r="H40" s="16" t="n"/>
-      <c r="I40" s="16" t="n"/>
+      <c r="G40" s="15" t="inlineStr">
+        <is>
+          <t>Hands On Kubernetes: "Project Lab: Scaling a Multi-Tier Web Application"</t>
+        </is>
+      </c>
+      <c r="H40" s="17" t="n"/>
+      <c r="I40" s="17" t="n"/>
+      <c r="J40" s="17" t="n"/>
     </row>
     <row r="41">
-      <c r="A41" s="17" t="n">
+      <c r="A41" s="16" t="n">
         <v>36</v>
       </c>
-      <c r="B41" s="17" t="n">
+      <c r="B41" s="16" t="n">
         <v>6</v>
       </c>
-      <c r="C41" s="17" t="inlineStr">
-        <is>
-          <t>Learn</t>
-        </is>
-      </c>
-      <c r="D41" s="17" t="inlineStr">
+      <c r="C41" s="16" t="inlineStr">
+        <is>
+          <t>Learn</t>
+        </is>
+      </c>
+      <c r="D41" s="16" t="inlineStr">
         <is>
           <t>CI/CD with GitHub Actions</t>
         </is>
       </c>
-      <c r="E41" s="17" t="inlineStr">
+      <c r="E41" s="16" t="inlineStr">
         <is>
           <t>Opens when Week 6 starts: see the Week 6 lesson. (CI/CD with GitHub Actions)</t>
         </is>
@@ -2367,28 +2555,33 @@
           <t>https://github.com/TechSckoolByVijay/75-day-career-upgrade/tree/main/week-06-cicd</t>
         </is>
       </c>
-      <c r="G41" s="16" t="n"/>
-      <c r="H41" s="16" t="n"/>
-      <c r="I41" s="16" t="n"/>
+      <c r="G41" s="15" t="inlineStr">
+        <is>
+          <t>Learning GitHub Actions for DevOps CI/CD: "the whole course; for the project: Building, Pushing &amp; Deploying Docker Containers"</t>
+        </is>
+      </c>
+      <c r="H41" s="17" t="n"/>
+      <c r="I41" s="17" t="n"/>
+      <c r="J41" s="17" t="n"/>
     </row>
     <row r="42">
-      <c r="A42" s="17" t="n">
+      <c r="A42" s="16" t="n">
         <v>37</v>
       </c>
-      <c r="B42" s="17" t="n">
+      <c r="B42" s="16" t="n">
         <v>6</v>
       </c>
-      <c r="C42" s="17" t="inlineStr">
-        <is>
-          <t>Learn</t>
-        </is>
-      </c>
-      <c r="D42" s="17" t="inlineStr">
+      <c r="C42" s="16" t="inlineStr">
+        <is>
+          <t>Learn</t>
+        </is>
+      </c>
+      <c r="D42" s="16" t="inlineStr">
         <is>
           <t>CI/CD with GitHub Actions</t>
         </is>
       </c>
-      <c r="E42" s="17" t="inlineStr">
+      <c r="E42" s="16" t="inlineStr">
         <is>
           <t>Opens when Week 6 starts: see the Week 6 lesson. (CI/CD with GitHub Actions)</t>
         </is>
@@ -2398,28 +2591,33 @@
           <t>https://github.com/TechSckoolByVijay/75-day-career-upgrade/tree/main/week-06-cicd</t>
         </is>
       </c>
-      <c r="G42" s="16" t="n"/>
-      <c r="H42" s="16" t="n"/>
-      <c r="I42" s="16" t="n"/>
+      <c r="G42" s="15" t="inlineStr">
+        <is>
+          <t>Learning GitHub Actions for DevOps CI/CD: "the whole course; for the project: Building, Pushing &amp; Deploying Docker Containers"</t>
+        </is>
+      </c>
+      <c r="H42" s="17" t="n"/>
+      <c r="I42" s="17" t="n"/>
+      <c r="J42" s="17" t="n"/>
     </row>
     <row r="43">
-      <c r="A43" s="17" t="n">
+      <c r="A43" s="16" t="n">
         <v>38</v>
       </c>
-      <c r="B43" s="17" t="n">
+      <c r="B43" s="16" t="n">
         <v>6</v>
       </c>
-      <c r="C43" s="17" t="inlineStr">
-        <is>
-          <t>Learn</t>
-        </is>
-      </c>
-      <c r="D43" s="17" t="inlineStr">
+      <c r="C43" s="16" t="inlineStr">
+        <is>
+          <t>Learn</t>
+        </is>
+      </c>
+      <c r="D43" s="16" t="inlineStr">
         <is>
           <t>CI/CD with GitHub Actions</t>
         </is>
       </c>
-      <c r="E43" s="17" t="inlineStr">
+      <c r="E43" s="16" t="inlineStr">
         <is>
           <t>Opens when Week 6 starts: see the Week 6 lesson. (CI/CD with GitHub Actions)</t>
         </is>
@@ -2429,28 +2627,33 @@
           <t>https://github.com/TechSckoolByVijay/75-day-career-upgrade/tree/main/week-06-cicd</t>
         </is>
       </c>
-      <c r="G43" s="16" t="n"/>
-      <c r="H43" s="16" t="n"/>
-      <c r="I43" s="16" t="n"/>
+      <c r="G43" s="15" t="inlineStr">
+        <is>
+          <t>Learning GitHub Actions for DevOps CI/CD: "the whole course; for the project: Building, Pushing &amp; Deploying Docker Containers"</t>
+        </is>
+      </c>
+      <c r="H43" s="17" t="n"/>
+      <c r="I43" s="17" t="n"/>
+      <c r="J43" s="17" t="n"/>
     </row>
     <row r="44">
-      <c r="A44" s="17" t="n">
+      <c r="A44" s="16" t="n">
         <v>39</v>
       </c>
-      <c r="B44" s="17" t="n">
+      <c r="B44" s="16" t="n">
         <v>6</v>
       </c>
-      <c r="C44" s="17" t="inlineStr">
-        <is>
-          <t>Learn</t>
-        </is>
-      </c>
-      <c r="D44" s="17" t="inlineStr">
+      <c r="C44" s="16" t="inlineStr">
+        <is>
+          <t>Learn</t>
+        </is>
+      </c>
+      <c r="D44" s="16" t="inlineStr">
         <is>
           <t>CI/CD with GitHub Actions</t>
         </is>
       </c>
-      <c r="E44" s="17" t="inlineStr">
+      <c r="E44" s="16" t="inlineStr">
         <is>
           <t>Opens when Week 6 starts: see the Week 6 lesson. (CI/CD with GitHub Actions)</t>
         </is>
@@ -2460,28 +2663,33 @@
           <t>https://github.com/TechSckoolByVijay/75-day-career-upgrade/tree/main/week-06-cicd</t>
         </is>
       </c>
-      <c r="G44" s="16" t="n"/>
-      <c r="H44" s="16" t="n"/>
-      <c r="I44" s="16" t="n"/>
+      <c r="G44" s="15" t="inlineStr">
+        <is>
+          <t>Learning GitHub Actions for DevOps CI/CD: "the whole course; for the project: Building, Pushing &amp; Deploying Docker Containers"</t>
+        </is>
+      </c>
+      <c r="H44" s="17" t="n"/>
+      <c r="I44" s="17" t="n"/>
+      <c r="J44" s="17" t="n"/>
     </row>
     <row r="45">
-      <c r="A45" s="17" t="n">
+      <c r="A45" s="16" t="n">
         <v>40</v>
       </c>
-      <c r="B45" s="17" t="n">
+      <c r="B45" s="16" t="n">
         <v>6</v>
       </c>
-      <c r="C45" s="17" t="inlineStr">
-        <is>
-          <t>Learn</t>
-        </is>
-      </c>
-      <c r="D45" s="17" t="inlineStr">
+      <c r="C45" s="16" t="inlineStr">
+        <is>
+          <t>Learn</t>
+        </is>
+      </c>
+      <c r="D45" s="16" t="inlineStr">
         <is>
           <t>CI/CD with GitHub Actions</t>
         </is>
       </c>
-      <c r="E45" s="17" t="inlineStr">
+      <c r="E45" s="16" t="inlineStr">
         <is>
           <t>Opens when Week 6 starts: see the Week 6 lesson. (CI/CD with GitHub Actions)</t>
         </is>
@@ -2491,9 +2699,14 @@
           <t>https://github.com/TechSckoolByVijay/75-day-career-upgrade/tree/main/week-06-cicd</t>
         </is>
       </c>
-      <c r="G45" s="16" t="n"/>
-      <c r="H45" s="16" t="n"/>
-      <c r="I45" s="16" t="n"/>
+      <c r="G45" s="15" t="inlineStr">
+        <is>
+          <t>Learning GitHub Actions for DevOps CI/CD: "the whole course; for the project: Building, Pushing &amp; Deploying Docker Containers"</t>
+        </is>
+      </c>
+      <c r="H45" s="17" t="n"/>
+      <c r="I45" s="17" t="n"/>
+      <c r="J45" s="17" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="14" t="n">
@@ -2522,9 +2735,14 @@
           <t>https://github.com/TechSckoolByVijay/75-day-career-upgrade/tree/main/week-06-cicd</t>
         </is>
       </c>
-      <c r="G46" s="16" t="n"/>
-      <c r="H46" s="16" t="n"/>
-      <c r="I46" s="16" t="n"/>
+      <c r="G46" s="15" t="inlineStr">
+        <is>
+          <t>Learning GitHub Actions for DevOps CI/CD: "the whole course; for the project: Building, Pushing &amp; Deploying Docker Containers"</t>
+        </is>
+      </c>
+      <c r="H46" s="17" t="n"/>
+      <c r="I46" s="17" t="n"/>
+      <c r="J46" s="17" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="14" t="n">
@@ -2553,28 +2771,33 @@
           <t>https://github.com/TechSckoolByVijay/75-day-career-upgrade/tree/main/week-06-cicd</t>
         </is>
       </c>
-      <c r="G47" s="16" t="n"/>
-      <c r="H47" s="16" t="n"/>
-      <c r="I47" s="16" t="n"/>
+      <c r="G47" s="15" t="inlineStr">
+        <is>
+          <t>Learning GitHub Actions for DevOps CI/CD: "the whole course; for the project: Building, Pushing &amp; Deploying Docker Containers"</t>
+        </is>
+      </c>
+      <c r="H47" s="17" t="n"/>
+      <c r="I47" s="17" t="n"/>
+      <c r="J47" s="17" t="n"/>
     </row>
     <row r="48">
-      <c r="A48" s="17" t="n">
+      <c r="A48" s="16" t="n">
         <v>43</v>
       </c>
-      <c r="B48" s="17" t="n">
+      <c r="B48" s="16" t="n">
         <v>7</v>
       </c>
-      <c r="C48" s="17" t="inlineStr">
-        <is>
-          <t>Learn</t>
-        </is>
-      </c>
-      <c r="D48" s="17" t="inlineStr">
+      <c r="C48" s="16" t="inlineStr">
+        <is>
+          <t>Learn</t>
+        </is>
+      </c>
+      <c r="D48" s="16" t="inlineStr">
         <is>
           <t>Cloud for admins (Azure)</t>
         </is>
       </c>
-      <c r="E48" s="17" t="inlineStr">
+      <c r="E48" s="16" t="inlineStr">
         <is>
           <t>Opens when Week 7 starts: see the Week 7 lesson. (Cloud for admins (Azure))</t>
         </is>
@@ -2584,28 +2807,33 @@
           <t>https://github.com/TechSckoolByVijay/75-day-career-upgrade/tree/main/week-07-cloud</t>
         </is>
       </c>
-      <c r="G48" s="16" t="n"/>
-      <c r="H48" s="16" t="n"/>
-      <c r="I48" s="16" t="n"/>
+      <c r="G48" s="15" t="inlineStr">
+        <is>
+          <t>AZ-900 Azure Fundamentals Quick Prep: "Core Azure services, identity, cost" · Learning Microsoft Azure: A Hands-On Training: "Projects 1-2: static website, website on a VM"</t>
+        </is>
+      </c>
+      <c r="H48" s="17" t="n"/>
+      <c r="I48" s="17" t="n"/>
+      <c r="J48" s="17" t="n"/>
     </row>
     <row r="49">
-      <c r="A49" s="17" t="n">
+      <c r="A49" s="16" t="n">
         <v>44</v>
       </c>
-      <c r="B49" s="17" t="n">
+      <c r="B49" s="16" t="n">
         <v>7</v>
       </c>
-      <c r="C49" s="17" t="inlineStr">
-        <is>
-          <t>Learn</t>
-        </is>
-      </c>
-      <c r="D49" s="17" t="inlineStr">
+      <c r="C49" s="16" t="inlineStr">
+        <is>
+          <t>Learn</t>
+        </is>
+      </c>
+      <c r="D49" s="16" t="inlineStr">
         <is>
           <t>Cloud for admins (Azure)</t>
         </is>
       </c>
-      <c r="E49" s="17" t="inlineStr">
+      <c r="E49" s="16" t="inlineStr">
         <is>
           <t>Opens when Week 7 starts: see the Week 7 lesson. (Cloud for admins (Azure))</t>
         </is>
@@ -2615,28 +2843,33 @@
           <t>https://github.com/TechSckoolByVijay/75-day-career-upgrade/tree/main/week-07-cloud</t>
         </is>
       </c>
-      <c r="G49" s="16" t="n"/>
-      <c r="H49" s="16" t="n"/>
-      <c r="I49" s="16" t="n"/>
+      <c r="G49" s="15" t="inlineStr">
+        <is>
+          <t>AZ-900 Azure Fundamentals Quick Prep: "Core Azure services, identity, cost" · Learning Microsoft Azure: A Hands-On Training: "Projects 1-2: static website, website on a VM"</t>
+        </is>
+      </c>
+      <c r="H49" s="17" t="n"/>
+      <c r="I49" s="17" t="n"/>
+      <c r="J49" s="17" t="n"/>
     </row>
     <row r="50">
-      <c r="A50" s="17" t="n">
+      <c r="A50" s="16" t="n">
         <v>45</v>
       </c>
-      <c r="B50" s="17" t="n">
+      <c r="B50" s="16" t="n">
         <v>7</v>
       </c>
-      <c r="C50" s="17" t="inlineStr">
-        <is>
-          <t>Learn</t>
-        </is>
-      </c>
-      <c r="D50" s="17" t="inlineStr">
+      <c r="C50" s="16" t="inlineStr">
+        <is>
+          <t>Learn</t>
+        </is>
+      </c>
+      <c r="D50" s="16" t="inlineStr">
         <is>
           <t>Cloud for admins (Azure)</t>
         </is>
       </c>
-      <c r="E50" s="17" t="inlineStr">
+      <c r="E50" s="16" t="inlineStr">
         <is>
           <t>Opens when Week 7 starts: see the Week 7 lesson. (Cloud for admins (Azure))</t>
         </is>
@@ -2646,28 +2879,33 @@
           <t>https://github.com/TechSckoolByVijay/75-day-career-upgrade/tree/main/week-07-cloud</t>
         </is>
       </c>
-      <c r="G50" s="16" t="n"/>
-      <c r="H50" s="16" t="n"/>
-      <c r="I50" s="16" t="n"/>
+      <c r="G50" s="15" t="inlineStr">
+        <is>
+          <t>AZ-900 Azure Fundamentals Quick Prep: "Core Azure services, identity, cost" · Learning Microsoft Azure: A Hands-On Training: "Projects 1-2: static website, website on a VM"</t>
+        </is>
+      </c>
+      <c r="H50" s="17" t="n"/>
+      <c r="I50" s="17" t="n"/>
+      <c r="J50" s="17" t="n"/>
     </row>
     <row r="51">
-      <c r="A51" s="17" t="n">
+      <c r="A51" s="16" t="n">
         <v>46</v>
       </c>
-      <c r="B51" s="17" t="n">
+      <c r="B51" s="16" t="n">
         <v>7</v>
       </c>
-      <c r="C51" s="17" t="inlineStr">
-        <is>
-          <t>Learn</t>
-        </is>
-      </c>
-      <c r="D51" s="17" t="inlineStr">
+      <c r="C51" s="16" t="inlineStr">
+        <is>
+          <t>Learn</t>
+        </is>
+      </c>
+      <c r="D51" s="16" t="inlineStr">
         <is>
           <t>Cloud for admins (Azure)</t>
         </is>
       </c>
-      <c r="E51" s="17" t="inlineStr">
+      <c r="E51" s="16" t="inlineStr">
         <is>
           <t>Opens when Week 7 starts: see the Week 7 lesson. (Cloud for admins (Azure))</t>
         </is>
@@ -2677,28 +2915,33 @@
           <t>https://github.com/TechSckoolByVijay/75-day-career-upgrade/tree/main/week-07-cloud</t>
         </is>
       </c>
-      <c r="G51" s="16" t="n"/>
-      <c r="H51" s="16" t="n"/>
-      <c r="I51" s="16" t="n"/>
+      <c r="G51" s="15" t="inlineStr">
+        <is>
+          <t>AZ-900 Azure Fundamentals Quick Prep: "Core Azure services, identity, cost" · Learning Microsoft Azure: A Hands-On Training: "Projects 1-2: static website, website on a VM"</t>
+        </is>
+      </c>
+      <c r="H51" s="17" t="n"/>
+      <c r="I51" s="17" t="n"/>
+      <c r="J51" s="17" t="n"/>
     </row>
     <row r="52">
-      <c r="A52" s="17" t="n">
+      <c r="A52" s="16" t="n">
         <v>47</v>
       </c>
-      <c r="B52" s="17" t="n">
+      <c r="B52" s="16" t="n">
         <v>7</v>
       </c>
-      <c r="C52" s="17" t="inlineStr">
-        <is>
-          <t>Learn</t>
-        </is>
-      </c>
-      <c r="D52" s="17" t="inlineStr">
+      <c r="C52" s="16" t="inlineStr">
+        <is>
+          <t>Learn</t>
+        </is>
+      </c>
+      <c r="D52" s="16" t="inlineStr">
         <is>
           <t>Cloud for admins (Azure)</t>
         </is>
       </c>
-      <c r="E52" s="17" t="inlineStr">
+      <c r="E52" s="16" t="inlineStr">
         <is>
           <t>Opens when Week 7 starts: see the Week 7 lesson. (Cloud for admins (Azure))</t>
         </is>
@@ -2708,9 +2951,14 @@
           <t>https://github.com/TechSckoolByVijay/75-day-career-upgrade/tree/main/week-07-cloud</t>
         </is>
       </c>
-      <c r="G52" s="16" t="n"/>
-      <c r="H52" s="16" t="n"/>
-      <c r="I52" s="16" t="n"/>
+      <c r="G52" s="15" t="inlineStr">
+        <is>
+          <t>AZ-900 Azure Fundamentals Quick Prep: "Core Azure services, identity, cost" · Learning Microsoft Azure: A Hands-On Training: "Projects 1-2: static website, website on a VM"</t>
+        </is>
+      </c>
+      <c r="H52" s="17" t="n"/>
+      <c r="I52" s="17" t="n"/>
+      <c r="J52" s="17" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="14" t="n">
@@ -2739,9 +2987,14 @@
           <t>https://github.com/TechSckoolByVijay/75-day-career-upgrade/tree/main/week-07-cloud</t>
         </is>
       </c>
-      <c r="G53" s="16" t="n"/>
-      <c r="H53" s="16" t="n"/>
-      <c r="I53" s="16" t="n"/>
+      <c r="G53" s="15" t="inlineStr">
+        <is>
+          <t>AZ-900 Azure Fundamentals Quick Prep: "Core Azure services, identity, cost" · Learning Microsoft Azure: A Hands-On Training: "Projects 1-2: static website, website on a VM"</t>
+        </is>
+      </c>
+      <c r="H53" s="17" t="n"/>
+      <c r="I53" s="17" t="n"/>
+      <c r="J53" s="17" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="14" t="n">
@@ -2770,28 +3023,33 @@
           <t>https://github.com/TechSckoolByVijay/75-day-career-upgrade/tree/main/week-07-cloud</t>
         </is>
       </c>
-      <c r="G54" s="16" t="n"/>
-      <c r="H54" s="16" t="n"/>
-      <c r="I54" s="16" t="n"/>
+      <c r="G54" s="15" t="inlineStr">
+        <is>
+          <t>AZ-900 Azure Fundamentals Quick Prep: "Core Azure services, identity, cost" · Learning Microsoft Azure: A Hands-On Training: "Projects 1-2: static website, website on a VM"</t>
+        </is>
+      </c>
+      <c r="H54" s="17" t="n"/>
+      <c r="I54" s="17" t="n"/>
+      <c r="J54" s="17" t="n"/>
     </row>
     <row r="55">
-      <c r="A55" s="17" t="n">
+      <c r="A55" s="16" t="n">
         <v>50</v>
       </c>
-      <c r="B55" s="17" t="n">
+      <c r="B55" s="16" t="n">
         <v>8</v>
       </c>
-      <c r="C55" s="17" t="inlineStr">
-        <is>
-          <t>Learn</t>
-        </is>
-      </c>
-      <c r="D55" s="17" t="inlineStr">
+      <c r="C55" s="16" t="inlineStr">
+        <is>
+          <t>Learn</t>
+        </is>
+      </c>
+      <c r="D55" s="16" t="inlineStr">
         <is>
           <t>Terraform (infrastructure as code)</t>
         </is>
       </c>
-      <c r="E55" s="17" t="inlineStr">
+      <c r="E55" s="16" t="inlineStr">
         <is>
           <t>Opens when Week 8 starts: see the Week 8 lesson. (Terraform (infrastructure as code))</t>
         </is>
@@ -2801,28 +3059,33 @@
           <t>https://github.com/TechSckoolByVijay/75-day-career-upgrade/tree/main/week-08-terraform</t>
         </is>
       </c>
-      <c r="G55" s="16" t="n"/>
-      <c r="H55" s="16" t="n"/>
-      <c r="I55" s="16" t="n"/>
+      <c r="G55" s="15" t="inlineStr">
+        <is>
+          <t>Terraform For GenAI DevOps Engineer: "Terraform Foundations &amp; Core Workflow; Variables, Dependencies &amp; State"</t>
+        </is>
+      </c>
+      <c r="H55" s="17" t="n"/>
+      <c r="I55" s="17" t="n"/>
+      <c r="J55" s="17" t="n"/>
     </row>
     <row r="56">
-      <c r="A56" s="17" t="n">
+      <c r="A56" s="16" t="n">
         <v>51</v>
       </c>
-      <c r="B56" s="17" t="n">
+      <c r="B56" s="16" t="n">
         <v>8</v>
       </c>
-      <c r="C56" s="17" t="inlineStr">
-        <is>
-          <t>Learn</t>
-        </is>
-      </c>
-      <c r="D56" s="17" t="inlineStr">
+      <c r="C56" s="16" t="inlineStr">
+        <is>
+          <t>Learn</t>
+        </is>
+      </c>
+      <c r="D56" s="16" t="inlineStr">
         <is>
           <t>Terraform (infrastructure as code)</t>
         </is>
       </c>
-      <c r="E56" s="17" t="inlineStr">
+      <c r="E56" s="16" t="inlineStr">
         <is>
           <t>Opens when Week 8 starts: see the Week 8 lesson. (Terraform (infrastructure as code))</t>
         </is>
@@ -2832,28 +3095,33 @@
           <t>https://github.com/TechSckoolByVijay/75-day-career-upgrade/tree/main/week-08-terraform</t>
         </is>
       </c>
-      <c r="G56" s="16" t="n"/>
-      <c r="H56" s="16" t="n"/>
-      <c r="I56" s="16" t="n"/>
+      <c r="G56" s="15" t="inlineStr">
+        <is>
+          <t>Terraform For GenAI DevOps Engineer: "Terraform Foundations &amp; Core Workflow; Variables, Dependencies &amp; State"</t>
+        </is>
+      </c>
+      <c r="H56" s="17" t="n"/>
+      <c r="I56" s="17" t="n"/>
+      <c r="J56" s="17" t="n"/>
     </row>
     <row r="57">
-      <c r="A57" s="17" t="n">
+      <c r="A57" s="16" t="n">
         <v>52</v>
       </c>
-      <c r="B57" s="17" t="n">
+      <c r="B57" s="16" t="n">
         <v>8</v>
       </c>
-      <c r="C57" s="17" t="inlineStr">
-        <is>
-          <t>Learn</t>
-        </is>
-      </c>
-      <c r="D57" s="17" t="inlineStr">
+      <c r="C57" s="16" t="inlineStr">
+        <is>
+          <t>Learn</t>
+        </is>
+      </c>
+      <c r="D57" s="16" t="inlineStr">
         <is>
           <t>Terraform (infrastructure as code)</t>
         </is>
       </c>
-      <c r="E57" s="17" t="inlineStr">
+      <c r="E57" s="16" t="inlineStr">
         <is>
           <t>Opens when Week 8 starts: see the Week 8 lesson. (Terraform (infrastructure as code))</t>
         </is>
@@ -2863,28 +3131,33 @@
           <t>https://github.com/TechSckoolByVijay/75-day-career-upgrade/tree/main/week-08-terraform</t>
         </is>
       </c>
-      <c r="G57" s="16" t="n"/>
-      <c r="H57" s="16" t="n"/>
-      <c r="I57" s="16" t="n"/>
+      <c r="G57" s="15" t="inlineStr">
+        <is>
+          <t>Terraform For GenAI DevOps Engineer: "Terraform Foundations &amp; Core Workflow; Variables, Dependencies &amp; State"</t>
+        </is>
+      </c>
+      <c r="H57" s="17" t="n"/>
+      <c r="I57" s="17" t="n"/>
+      <c r="J57" s="17" t="n"/>
     </row>
     <row r="58">
-      <c r="A58" s="17" t="n">
+      <c r="A58" s="16" t="n">
         <v>53</v>
       </c>
-      <c r="B58" s="17" t="n">
+      <c r="B58" s="16" t="n">
         <v>8</v>
       </c>
-      <c r="C58" s="17" t="inlineStr">
-        <is>
-          <t>Learn</t>
-        </is>
-      </c>
-      <c r="D58" s="17" t="inlineStr">
+      <c r="C58" s="16" t="inlineStr">
+        <is>
+          <t>Learn</t>
+        </is>
+      </c>
+      <c r="D58" s="16" t="inlineStr">
         <is>
           <t>Terraform (infrastructure as code)</t>
         </is>
       </c>
-      <c r="E58" s="17" t="inlineStr">
+      <c r="E58" s="16" t="inlineStr">
         <is>
           <t>Opens when Week 8 starts: see the Week 8 lesson. (Terraform (infrastructure as code))</t>
         </is>
@@ -2894,28 +3167,33 @@
           <t>https://github.com/TechSckoolByVijay/75-day-career-upgrade/tree/main/week-08-terraform</t>
         </is>
       </c>
-      <c r="G58" s="16" t="n"/>
-      <c r="H58" s="16" t="n"/>
-      <c r="I58" s="16" t="n"/>
+      <c r="G58" s="15" t="inlineStr">
+        <is>
+          <t>Terraform For GenAI DevOps Engineer: "Terraform Foundations &amp; Core Workflow; Variables, Dependencies &amp; State"</t>
+        </is>
+      </c>
+      <c r="H58" s="17" t="n"/>
+      <c r="I58" s="17" t="n"/>
+      <c r="J58" s="17" t="n"/>
     </row>
     <row r="59">
-      <c r="A59" s="17" t="n">
+      <c r="A59" s="16" t="n">
         <v>54</v>
       </c>
-      <c r="B59" s="17" t="n">
+      <c r="B59" s="16" t="n">
         <v>8</v>
       </c>
-      <c r="C59" s="17" t="inlineStr">
-        <is>
-          <t>Learn</t>
-        </is>
-      </c>
-      <c r="D59" s="17" t="inlineStr">
+      <c r="C59" s="16" t="inlineStr">
+        <is>
+          <t>Learn</t>
+        </is>
+      </c>
+      <c r="D59" s="16" t="inlineStr">
         <is>
           <t>Terraform (infrastructure as code)</t>
         </is>
       </c>
-      <c r="E59" s="17" t="inlineStr">
+      <c r="E59" s="16" t="inlineStr">
         <is>
           <t>Opens when Week 8 starts: see the Week 8 lesson. (Terraform (infrastructure as code))</t>
         </is>
@@ -2925,9 +3203,14 @@
           <t>https://github.com/TechSckoolByVijay/75-day-career-upgrade/tree/main/week-08-terraform</t>
         </is>
       </c>
-      <c r="G59" s="16" t="n"/>
-      <c r="H59" s="16" t="n"/>
-      <c r="I59" s="16" t="n"/>
+      <c r="G59" s="15" t="inlineStr">
+        <is>
+          <t>Terraform For GenAI DevOps Engineer: "Terraform Foundations &amp; Core Workflow; Variables, Dependencies &amp; State"</t>
+        </is>
+      </c>
+      <c r="H59" s="17" t="n"/>
+      <c r="I59" s="17" t="n"/>
+      <c r="J59" s="17" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="14" t="n">
@@ -2956,9 +3239,14 @@
           <t>https://github.com/TechSckoolByVijay/75-day-career-upgrade/tree/main/week-08-terraform</t>
         </is>
       </c>
-      <c r="G60" s="16" t="n"/>
-      <c r="H60" s="16" t="n"/>
-      <c r="I60" s="16" t="n"/>
+      <c r="G60" s="15" t="inlineStr">
+        <is>
+          <t>Terraform For GenAI DevOps Engineer: "Terraform Foundations &amp; Core Workflow; Variables, Dependencies &amp; State"</t>
+        </is>
+      </c>
+      <c r="H60" s="17" t="n"/>
+      <c r="I60" s="17" t="n"/>
+      <c r="J60" s="17" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="14" t="n">
@@ -2987,28 +3275,33 @@
           <t>https://github.com/TechSckoolByVijay/75-day-career-upgrade/tree/main/week-08-terraform</t>
         </is>
       </c>
-      <c r="G61" s="16" t="n"/>
-      <c r="H61" s="16" t="n"/>
-      <c r="I61" s="16" t="n"/>
+      <c r="G61" s="15" t="inlineStr">
+        <is>
+          <t>Terraform For GenAI DevOps Engineer: "Terraform Foundations &amp; Core Workflow; Variables, Dependencies &amp; State"</t>
+        </is>
+      </c>
+      <c r="H61" s="17" t="n"/>
+      <c r="I61" s="17" t="n"/>
+      <c r="J61" s="17" t="n"/>
     </row>
     <row r="62">
-      <c r="A62" s="17" t="n">
+      <c r="A62" s="16" t="n">
         <v>57</v>
       </c>
-      <c r="B62" s="17" t="n">
+      <c r="B62" s="16" t="n">
         <v>9</v>
       </c>
-      <c r="C62" s="17" t="inlineStr">
-        <is>
-          <t>Learn</t>
-        </is>
-      </c>
-      <c r="D62" s="17" t="inlineStr">
+      <c r="C62" s="16" t="inlineStr">
+        <is>
+          <t>Learn</t>
+        </is>
+      </c>
+      <c r="D62" s="16" t="inlineStr">
         <is>
           <t>Checkpoint 2: end-to-end project</t>
         </is>
       </c>
-      <c r="E62" s="17" t="inlineStr">
+      <c r="E62" s="16" t="inlineStr">
         <is>
           <t>Opens when Week 9 starts: see the Week 9 lesson. (Checkpoint 2: end-to-end project)</t>
         </is>
@@ -3018,28 +3311,33 @@
           <t>https://github.com/TechSckoolByVijay/75-day-career-upgrade/tree/main/week-09-checkpoint-2</t>
         </is>
       </c>
-      <c r="G62" s="16" t="n"/>
-      <c r="H62" s="16" t="n"/>
-      <c r="I62" s="16" t="n"/>
+      <c r="G62" s="15" t="inlineStr">
+        <is>
+          <t>Learning GitHub Actions for DevOps CI/CD: "Building, Pushing &amp; Deploying Docker Containers" · Terraform For GenAI DevOps Engineer: "Migrating tfstate to Remote Backend"</t>
+        </is>
+      </c>
+      <c r="H62" s="17" t="n"/>
+      <c r="I62" s="17" t="n"/>
+      <c r="J62" s="17" t="n"/>
     </row>
     <row r="63">
-      <c r="A63" s="17" t="n">
+      <c r="A63" s="16" t="n">
         <v>58</v>
       </c>
-      <c r="B63" s="17" t="n">
+      <c r="B63" s="16" t="n">
         <v>9</v>
       </c>
-      <c r="C63" s="17" t="inlineStr">
-        <is>
-          <t>Learn</t>
-        </is>
-      </c>
-      <c r="D63" s="17" t="inlineStr">
+      <c r="C63" s="16" t="inlineStr">
+        <is>
+          <t>Learn</t>
+        </is>
+      </c>
+      <c r="D63" s="16" t="inlineStr">
         <is>
           <t>Checkpoint 2: end-to-end project</t>
         </is>
       </c>
-      <c r="E63" s="17" t="inlineStr">
+      <c r="E63" s="16" t="inlineStr">
         <is>
           <t>Opens when Week 9 starts: see the Week 9 lesson. (Checkpoint 2: end-to-end project)</t>
         </is>
@@ -3049,28 +3347,33 @@
           <t>https://github.com/TechSckoolByVijay/75-day-career-upgrade/tree/main/week-09-checkpoint-2</t>
         </is>
       </c>
-      <c r="G63" s="16" t="n"/>
-      <c r="H63" s="16" t="n"/>
-      <c r="I63" s="16" t="n"/>
+      <c r="G63" s="15" t="inlineStr">
+        <is>
+          <t>Learning GitHub Actions for DevOps CI/CD: "Building, Pushing &amp; Deploying Docker Containers" · Terraform For GenAI DevOps Engineer: "Migrating tfstate to Remote Backend"</t>
+        </is>
+      </c>
+      <c r="H63" s="17" t="n"/>
+      <c r="I63" s="17" t="n"/>
+      <c r="J63" s="17" t="n"/>
     </row>
     <row r="64">
-      <c r="A64" s="17" t="n">
+      <c r="A64" s="16" t="n">
         <v>59</v>
       </c>
-      <c r="B64" s="17" t="n">
+      <c r="B64" s="16" t="n">
         <v>9</v>
       </c>
-      <c r="C64" s="17" t="inlineStr">
-        <is>
-          <t>Learn</t>
-        </is>
-      </c>
-      <c r="D64" s="17" t="inlineStr">
+      <c r="C64" s="16" t="inlineStr">
+        <is>
+          <t>Learn</t>
+        </is>
+      </c>
+      <c r="D64" s="16" t="inlineStr">
         <is>
           <t>Checkpoint 2: end-to-end project</t>
         </is>
       </c>
-      <c r="E64" s="17" t="inlineStr">
+      <c r="E64" s="16" t="inlineStr">
         <is>
           <t>Opens when Week 9 starts: see the Week 9 lesson. (Checkpoint 2: end-to-end project)</t>
         </is>
@@ -3080,28 +3383,33 @@
           <t>https://github.com/TechSckoolByVijay/75-day-career-upgrade/tree/main/week-09-checkpoint-2</t>
         </is>
       </c>
-      <c r="G64" s="16" t="n"/>
-      <c r="H64" s="16" t="n"/>
-      <c r="I64" s="16" t="n"/>
+      <c r="G64" s="15" t="inlineStr">
+        <is>
+          <t>Learning GitHub Actions for DevOps CI/CD: "Building, Pushing &amp; Deploying Docker Containers" · Terraform For GenAI DevOps Engineer: "Migrating tfstate to Remote Backend"</t>
+        </is>
+      </c>
+      <c r="H64" s="17" t="n"/>
+      <c r="I64" s="17" t="n"/>
+      <c r="J64" s="17" t="n"/>
     </row>
     <row r="65">
-      <c r="A65" s="17" t="n">
+      <c r="A65" s="16" t="n">
         <v>60</v>
       </c>
-      <c r="B65" s="17" t="n">
+      <c r="B65" s="16" t="n">
         <v>9</v>
       </c>
-      <c r="C65" s="17" t="inlineStr">
-        <is>
-          <t>Learn</t>
-        </is>
-      </c>
-      <c r="D65" s="17" t="inlineStr">
+      <c r="C65" s="16" t="inlineStr">
+        <is>
+          <t>Learn</t>
+        </is>
+      </c>
+      <c r="D65" s="16" t="inlineStr">
         <is>
           <t>Checkpoint 2: end-to-end project</t>
         </is>
       </c>
-      <c r="E65" s="17" t="inlineStr">
+      <c r="E65" s="16" t="inlineStr">
         <is>
           <t>Opens when Week 9 starts: see the Week 9 lesson. (Checkpoint 2: end-to-end project)</t>
         </is>
@@ -3111,28 +3419,33 @@
           <t>https://github.com/TechSckoolByVijay/75-day-career-upgrade/tree/main/week-09-checkpoint-2</t>
         </is>
       </c>
-      <c r="G65" s="16" t="n"/>
-      <c r="H65" s="16" t="n"/>
-      <c r="I65" s="16" t="n"/>
+      <c r="G65" s="15" t="inlineStr">
+        <is>
+          <t>Learning GitHub Actions for DevOps CI/CD: "Building, Pushing &amp; Deploying Docker Containers" · Terraform For GenAI DevOps Engineer: "Migrating tfstate to Remote Backend"</t>
+        </is>
+      </c>
+      <c r="H65" s="17" t="n"/>
+      <c r="I65" s="17" t="n"/>
+      <c r="J65" s="17" t="n"/>
     </row>
     <row r="66">
-      <c r="A66" s="17" t="n">
+      <c r="A66" s="16" t="n">
         <v>61</v>
       </c>
-      <c r="B66" s="17" t="n">
+      <c r="B66" s="16" t="n">
         <v>9</v>
       </c>
-      <c r="C66" s="17" t="inlineStr">
-        <is>
-          <t>Learn</t>
-        </is>
-      </c>
-      <c r="D66" s="17" t="inlineStr">
+      <c r="C66" s="16" t="inlineStr">
+        <is>
+          <t>Learn</t>
+        </is>
+      </c>
+      <c r="D66" s="16" t="inlineStr">
         <is>
           <t>Checkpoint 2: end-to-end project</t>
         </is>
       </c>
-      <c r="E66" s="17" t="inlineStr">
+      <c r="E66" s="16" t="inlineStr">
         <is>
           <t>Opens when Week 9 starts: see the Week 9 lesson. (Checkpoint 2: end-to-end project)</t>
         </is>
@@ -3142,9 +3455,14 @@
           <t>https://github.com/TechSckoolByVijay/75-day-career-upgrade/tree/main/week-09-checkpoint-2</t>
         </is>
       </c>
-      <c r="G66" s="16" t="n"/>
-      <c r="H66" s="16" t="n"/>
-      <c r="I66" s="16" t="n"/>
+      <c r="G66" s="15" t="inlineStr">
+        <is>
+          <t>Learning GitHub Actions for DevOps CI/CD: "Building, Pushing &amp; Deploying Docker Containers" · Terraform For GenAI DevOps Engineer: "Migrating tfstate to Remote Backend"</t>
+        </is>
+      </c>
+      <c r="H66" s="17" t="n"/>
+      <c r="I66" s="17" t="n"/>
+      <c r="J66" s="17" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="14" t="n">
@@ -3173,9 +3491,14 @@
           <t>https://github.com/TechSckoolByVijay/75-day-career-upgrade/tree/main/week-09-checkpoint-2</t>
         </is>
       </c>
-      <c r="G67" s="16" t="n"/>
-      <c r="H67" s="16" t="n"/>
-      <c r="I67" s="16" t="n"/>
+      <c r="G67" s="15" t="inlineStr">
+        <is>
+          <t>Learning GitHub Actions for DevOps CI/CD: "Building, Pushing &amp; Deploying Docker Containers" · Terraform For GenAI DevOps Engineer: "Migrating tfstate to Remote Backend"</t>
+        </is>
+      </c>
+      <c r="H67" s="17" t="n"/>
+      <c r="I67" s="17" t="n"/>
+      <c r="J67" s="17" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="14" t="n">
@@ -3204,28 +3527,33 @@
           <t>https://github.com/TechSckoolByVijay/75-day-career-upgrade/tree/main/week-09-checkpoint-2</t>
         </is>
       </c>
-      <c r="G68" s="16" t="n"/>
-      <c r="H68" s="16" t="n"/>
-      <c r="I68" s="16" t="n"/>
+      <c r="G68" s="15" t="inlineStr">
+        <is>
+          <t>Learning GitHub Actions for DevOps CI/CD: "Building, Pushing &amp; Deploying Docker Containers" · Terraform For GenAI DevOps Engineer: "Migrating tfstate to Remote Backend"</t>
+        </is>
+      </c>
+      <c r="H68" s="17" t="n"/>
+      <c r="I68" s="17" t="n"/>
+      <c r="J68" s="17" t="n"/>
     </row>
     <row r="69">
-      <c r="A69" s="17" t="n">
+      <c r="A69" s="16" t="n">
         <v>64</v>
       </c>
-      <c r="B69" s="17" t="n">
+      <c r="B69" s="16" t="n">
         <v>10</v>
       </c>
-      <c r="C69" s="17" t="inlineStr">
-        <is>
-          <t>Learn</t>
-        </is>
-      </c>
-      <c r="D69" s="17" t="inlineStr">
+      <c r="C69" s="16" t="inlineStr">
+        <is>
+          <t>Learn</t>
+        </is>
+      </c>
+      <c r="D69" s="16" t="inlineStr">
         <is>
           <t>AI in DevOps and SRE</t>
         </is>
       </c>
-      <c r="E69" s="17" t="inlineStr">
+      <c r="E69" s="16" t="inlineStr">
         <is>
           <t>Opens when Week 10 starts: see the Week 10 lesson. (AI in DevOps and SRE)</t>
         </is>
@@ -3235,28 +3563,33 @@
           <t>https://github.com/TechSckoolByVijay/75-day-career-upgrade/tree/main/week-10-ai-devops-sre</t>
         </is>
       </c>
-      <c r="G69" s="16" t="n"/>
-      <c r="H69" s="16" t="n"/>
-      <c r="I69" s="16" t="n"/>
+      <c r="G69" s="15" t="inlineStr">
+        <is>
+          <t>ChatGPT for DevOps: "the whole course" · k8s Production Readiness: "Building Secret-less GenAI Applications with Azure Workload Identity" · n8n Masterclass: Build a GenAI News Factory: "optional: AI agents and automation"</t>
+        </is>
+      </c>
+      <c r="H69" s="17" t="n"/>
+      <c r="I69" s="17" t="n"/>
+      <c r="J69" s="17" t="n"/>
     </row>
     <row r="70">
-      <c r="A70" s="17" t="n">
+      <c r="A70" s="16" t="n">
         <v>65</v>
       </c>
-      <c r="B70" s="17" t="n">
+      <c r="B70" s="16" t="n">
         <v>10</v>
       </c>
-      <c r="C70" s="17" t="inlineStr">
-        <is>
-          <t>Learn</t>
-        </is>
-      </c>
-      <c r="D70" s="17" t="inlineStr">
+      <c r="C70" s="16" t="inlineStr">
+        <is>
+          <t>Learn</t>
+        </is>
+      </c>
+      <c r="D70" s="16" t="inlineStr">
         <is>
           <t>AI in DevOps and SRE</t>
         </is>
       </c>
-      <c r="E70" s="17" t="inlineStr">
+      <c r="E70" s="16" t="inlineStr">
         <is>
           <t>Opens when Week 10 starts: see the Week 10 lesson. (AI in DevOps and SRE)</t>
         </is>
@@ -3266,28 +3599,33 @@
           <t>https://github.com/TechSckoolByVijay/75-day-career-upgrade/tree/main/week-10-ai-devops-sre</t>
         </is>
       </c>
-      <c r="G70" s="16" t="n"/>
-      <c r="H70" s="16" t="n"/>
-      <c r="I70" s="16" t="n"/>
+      <c r="G70" s="15" t="inlineStr">
+        <is>
+          <t>ChatGPT for DevOps: "the whole course" · k8s Production Readiness: "Building Secret-less GenAI Applications with Azure Workload Identity" · n8n Masterclass: Build a GenAI News Factory: "optional: AI agents and automation"</t>
+        </is>
+      </c>
+      <c r="H70" s="17" t="n"/>
+      <c r="I70" s="17" t="n"/>
+      <c r="J70" s="17" t="n"/>
     </row>
     <row r="71">
-      <c r="A71" s="17" t="n">
+      <c r="A71" s="16" t="n">
         <v>66</v>
       </c>
-      <c r="B71" s="17" t="n">
+      <c r="B71" s="16" t="n">
         <v>10</v>
       </c>
-      <c r="C71" s="17" t="inlineStr">
-        <is>
-          <t>Learn</t>
-        </is>
-      </c>
-      <c r="D71" s="17" t="inlineStr">
+      <c r="C71" s="16" t="inlineStr">
+        <is>
+          <t>Learn</t>
+        </is>
+      </c>
+      <c r="D71" s="16" t="inlineStr">
         <is>
           <t>AI in DevOps and SRE</t>
         </is>
       </c>
-      <c r="E71" s="17" t="inlineStr">
+      <c r="E71" s="16" t="inlineStr">
         <is>
           <t>Opens when Week 10 starts: see the Week 10 lesson. (AI in DevOps and SRE)</t>
         </is>
@@ -3297,28 +3635,33 @@
           <t>https://github.com/TechSckoolByVijay/75-day-career-upgrade/tree/main/week-10-ai-devops-sre</t>
         </is>
       </c>
-      <c r="G71" s="16" t="n"/>
-      <c r="H71" s="16" t="n"/>
-      <c r="I71" s="16" t="n"/>
+      <c r="G71" s="15" t="inlineStr">
+        <is>
+          <t>ChatGPT for DevOps: "the whole course" · k8s Production Readiness: "Building Secret-less GenAI Applications with Azure Workload Identity" · n8n Masterclass: Build a GenAI News Factory: "optional: AI agents and automation"</t>
+        </is>
+      </c>
+      <c r="H71" s="17" t="n"/>
+      <c r="I71" s="17" t="n"/>
+      <c r="J71" s="17" t="n"/>
     </row>
     <row r="72">
-      <c r="A72" s="17" t="n">
+      <c r="A72" s="16" t="n">
         <v>67</v>
       </c>
-      <c r="B72" s="17" t="n">
+      <c r="B72" s="16" t="n">
         <v>10</v>
       </c>
-      <c r="C72" s="17" t="inlineStr">
-        <is>
-          <t>Learn</t>
-        </is>
-      </c>
-      <c r="D72" s="17" t="inlineStr">
+      <c r="C72" s="16" t="inlineStr">
+        <is>
+          <t>Learn</t>
+        </is>
+      </c>
+      <c r="D72" s="16" t="inlineStr">
         <is>
           <t>AI in DevOps and SRE</t>
         </is>
       </c>
-      <c r="E72" s="17" t="inlineStr">
+      <c r="E72" s="16" t="inlineStr">
         <is>
           <t>Opens when Week 10 starts: see the Week 10 lesson. (AI in DevOps and SRE)</t>
         </is>
@@ -3328,28 +3671,33 @@
           <t>https://github.com/TechSckoolByVijay/75-day-career-upgrade/tree/main/week-10-ai-devops-sre</t>
         </is>
       </c>
-      <c r="G72" s="16" t="n"/>
-      <c r="H72" s="16" t="n"/>
-      <c r="I72" s="16" t="n"/>
+      <c r="G72" s="15" t="inlineStr">
+        <is>
+          <t>ChatGPT for DevOps: "the whole course" · k8s Production Readiness: "Building Secret-less GenAI Applications with Azure Workload Identity" · n8n Masterclass: Build a GenAI News Factory: "optional: AI agents and automation"</t>
+        </is>
+      </c>
+      <c r="H72" s="17" t="n"/>
+      <c r="I72" s="17" t="n"/>
+      <c r="J72" s="17" t="n"/>
     </row>
     <row r="73">
-      <c r="A73" s="17" t="n">
+      <c r="A73" s="16" t="n">
         <v>68</v>
       </c>
-      <c r="B73" s="17" t="n">
+      <c r="B73" s="16" t="n">
         <v>10</v>
       </c>
-      <c r="C73" s="17" t="inlineStr">
-        <is>
-          <t>Learn</t>
-        </is>
-      </c>
-      <c r="D73" s="17" t="inlineStr">
+      <c r="C73" s="16" t="inlineStr">
+        <is>
+          <t>Learn</t>
+        </is>
+      </c>
+      <c r="D73" s="16" t="inlineStr">
         <is>
           <t>AI in DevOps and SRE</t>
         </is>
       </c>
-      <c r="E73" s="17" t="inlineStr">
+      <c r="E73" s="16" t="inlineStr">
         <is>
           <t>Opens when Week 10 starts: see the Week 10 lesson. (AI in DevOps and SRE)</t>
         </is>
@@ -3359,9 +3707,14 @@
           <t>https://github.com/TechSckoolByVijay/75-day-career-upgrade/tree/main/week-10-ai-devops-sre</t>
         </is>
       </c>
-      <c r="G73" s="16" t="n"/>
-      <c r="H73" s="16" t="n"/>
-      <c r="I73" s="16" t="n"/>
+      <c r="G73" s="15" t="inlineStr">
+        <is>
+          <t>ChatGPT for DevOps: "the whole course" · k8s Production Readiness: "Building Secret-less GenAI Applications with Azure Workload Identity" · n8n Masterclass: Build a GenAI News Factory: "optional: AI agents and automation"</t>
+        </is>
+      </c>
+      <c r="H73" s="17" t="n"/>
+      <c r="I73" s="17" t="n"/>
+      <c r="J73" s="17" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="14" t="n">
@@ -3390,9 +3743,14 @@
           <t>https://github.com/TechSckoolByVijay/75-day-career-upgrade/tree/main/week-10-ai-devops-sre</t>
         </is>
       </c>
-      <c r="G74" s="16" t="n"/>
-      <c r="H74" s="16" t="n"/>
-      <c r="I74" s="16" t="n"/>
+      <c r="G74" s="15" t="inlineStr">
+        <is>
+          <t>ChatGPT for DevOps: "the whole course" · k8s Production Readiness: "Building Secret-less GenAI Applications with Azure Workload Identity" · n8n Masterclass: Build a GenAI News Factory: "optional: AI agents and automation"</t>
+        </is>
+      </c>
+      <c r="H74" s="17" t="n"/>
+      <c r="I74" s="17" t="n"/>
+      <c r="J74" s="17" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="14" t="n">
@@ -3421,28 +3779,33 @@
           <t>https://github.com/TechSckoolByVijay/75-day-career-upgrade/tree/main/week-10-ai-devops-sre</t>
         </is>
       </c>
-      <c r="G75" s="16" t="n"/>
-      <c r="H75" s="16" t="n"/>
-      <c r="I75" s="16" t="n"/>
+      <c r="G75" s="15" t="inlineStr">
+        <is>
+          <t>ChatGPT for DevOps: "the whole course" · k8s Production Readiness: "Building Secret-less GenAI Applications with Azure Workload Identity" · n8n Masterclass: Build a GenAI News Factory: "optional: AI agents and automation"</t>
+        </is>
+      </c>
+      <c r="H75" s="17" t="n"/>
+      <c r="I75" s="17" t="n"/>
+      <c r="J75" s="17" t="n"/>
     </row>
     <row r="76">
-      <c r="A76" s="17" t="n">
+      <c r="A76" s="16" t="n">
         <v>71</v>
       </c>
-      <c r="B76" s="17" t="n">
+      <c r="B76" s="16" t="n">
         <v>11</v>
       </c>
-      <c r="C76" s="17" t="inlineStr">
-        <is>
-          <t>Learn</t>
-        </is>
-      </c>
-      <c r="D76" s="17" t="inlineStr">
+      <c r="C76" s="16" t="inlineStr">
+        <is>
+          <t>Learn</t>
+        </is>
+      </c>
+      <c r="D76" s="16" t="inlineStr">
         <is>
           <t>Capstone + pick your path</t>
         </is>
       </c>
-      <c r="E76" s="17" t="inlineStr">
+      <c r="E76" s="16" t="inlineStr">
         <is>
           <t>Opens when Week 11 starts: see the Week 11 lesson. (Capstone + pick your path)</t>
         </is>
@@ -3452,28 +3815,33 @@
           <t>https://github.com/TechSckoolByVijay/75-day-career-upgrade/tree/main/week-11-capstone</t>
         </is>
       </c>
-      <c r="G76" s="16" t="n"/>
-      <c r="H76" s="16" t="n"/>
-      <c r="I76" s="16" t="n"/>
+      <c r="G76" s="15" t="inlineStr">
+        <is>
+          <t>Everything above, at the challenge price: the AI-Enabled DevOps &amp; SRE bundle</t>
+        </is>
+      </c>
+      <c r="H76" s="17" t="n"/>
+      <c r="I76" s="17" t="n"/>
+      <c r="J76" s="17" t="n"/>
     </row>
     <row r="77">
-      <c r="A77" s="17" t="n">
+      <c r="A77" s="16" t="n">
         <v>72</v>
       </c>
-      <c r="B77" s="17" t="n">
+      <c r="B77" s="16" t="n">
         <v>11</v>
       </c>
-      <c r="C77" s="17" t="inlineStr">
-        <is>
-          <t>Learn</t>
-        </is>
-      </c>
-      <c r="D77" s="17" t="inlineStr">
+      <c r="C77" s="16" t="inlineStr">
+        <is>
+          <t>Learn</t>
+        </is>
+      </c>
+      <c r="D77" s="16" t="inlineStr">
         <is>
           <t>Capstone + pick your path</t>
         </is>
       </c>
-      <c r="E77" s="17" t="inlineStr">
+      <c r="E77" s="16" t="inlineStr">
         <is>
           <t>Opens when Week 11 starts: see the Week 11 lesson. (Capstone + pick your path)</t>
         </is>
@@ -3483,28 +3851,33 @@
           <t>https://github.com/TechSckoolByVijay/75-day-career-upgrade/tree/main/week-11-capstone</t>
         </is>
       </c>
-      <c r="G77" s="16" t="n"/>
-      <c r="H77" s="16" t="n"/>
-      <c r="I77" s="16" t="n"/>
+      <c r="G77" s="15" t="inlineStr">
+        <is>
+          <t>Everything above, at the challenge price: the AI-Enabled DevOps &amp; SRE bundle</t>
+        </is>
+      </c>
+      <c r="H77" s="17" t="n"/>
+      <c r="I77" s="17" t="n"/>
+      <c r="J77" s="17" t="n"/>
     </row>
     <row r="78">
-      <c r="A78" s="17" t="n">
+      <c r="A78" s="16" t="n">
         <v>73</v>
       </c>
-      <c r="B78" s="17" t="n">
+      <c r="B78" s="16" t="n">
         <v>11</v>
       </c>
-      <c r="C78" s="17" t="inlineStr">
-        <is>
-          <t>Learn</t>
-        </is>
-      </c>
-      <c r="D78" s="17" t="inlineStr">
+      <c r="C78" s="16" t="inlineStr">
+        <is>
+          <t>Learn</t>
+        </is>
+      </c>
+      <c r="D78" s="16" t="inlineStr">
         <is>
           <t>Capstone + pick your path</t>
         </is>
       </c>
-      <c r="E78" s="17" t="inlineStr">
+      <c r="E78" s="16" t="inlineStr">
         <is>
           <t>Opens when Week 11 starts: see the Week 11 lesson. (Capstone + pick your path)</t>
         </is>
@@ -3514,28 +3887,33 @@
           <t>https://github.com/TechSckoolByVijay/75-day-career-upgrade/tree/main/week-11-capstone</t>
         </is>
       </c>
-      <c r="G78" s="16" t="n"/>
-      <c r="H78" s="16" t="n"/>
-      <c r="I78" s="16" t="n"/>
+      <c r="G78" s="15" t="inlineStr">
+        <is>
+          <t>Everything above, at the challenge price: the AI-Enabled DevOps &amp; SRE bundle</t>
+        </is>
+      </c>
+      <c r="H78" s="17" t="n"/>
+      <c r="I78" s="17" t="n"/>
+      <c r="J78" s="17" t="n"/>
     </row>
     <row r="79">
-      <c r="A79" s="17" t="n">
+      <c r="A79" s="16" t="n">
         <v>74</v>
       </c>
-      <c r="B79" s="17" t="n">
+      <c r="B79" s="16" t="n">
         <v>11</v>
       </c>
-      <c r="C79" s="17" t="inlineStr">
-        <is>
-          <t>Learn</t>
-        </is>
-      </c>
-      <c r="D79" s="17" t="inlineStr">
+      <c r="C79" s="16" t="inlineStr">
+        <is>
+          <t>Learn</t>
+        </is>
+      </c>
+      <c r="D79" s="16" t="inlineStr">
         <is>
           <t>Capstone + pick your path</t>
         </is>
       </c>
-      <c r="E79" s="17" t="inlineStr">
+      <c r="E79" s="16" t="inlineStr">
         <is>
           <t>Opens when Week 11 starts: see the Week 11 lesson. (Capstone + pick your path)</t>
         </is>
@@ -3545,9 +3923,14 @@
           <t>https://github.com/TechSckoolByVijay/75-day-career-upgrade/tree/main/week-11-capstone</t>
         </is>
       </c>
-      <c r="G79" s="16" t="n"/>
-      <c r="H79" s="16" t="n"/>
-      <c r="I79" s="16" t="n"/>
+      <c r="G79" s="15" t="inlineStr">
+        <is>
+          <t>Everything above, at the challenge price: the AI-Enabled DevOps &amp; SRE bundle</t>
+        </is>
+      </c>
+      <c r="H79" s="17" t="n"/>
+      <c r="I79" s="17" t="n"/>
+      <c r="J79" s="17" t="n"/>
     </row>
     <row r="80">
       <c r="A80" s="14" t="n">
@@ -3576,28 +3959,33 @@
           <t>https://github.com/TechSckoolByVijay/75-day-career-upgrade/tree/main/week-11-capstone</t>
         </is>
       </c>
-      <c r="G80" s="16" t="n"/>
-      <c r="H80" s="16" t="n"/>
-      <c r="I80" s="16" t="n"/>
+      <c r="G80" s="15" t="inlineStr">
+        <is>
+          <t>Everything above, at the challenge price: the AI-Enabled DevOps &amp; SRE bundle</t>
+        </is>
+      </c>
+      <c r="H80" s="17" t="n"/>
+      <c r="I80" s="17" t="n"/>
+      <c r="J80" s="17" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I80"/>
-  <conditionalFormatting sqref="G2:G80">
+  <autoFilter ref="A1:J80"/>
+  <conditionalFormatting sqref="H2:H80">
     <cfRule type="expression" priority="1" dxfId="0">
-      <formula>$G2="Yes"</formula>
+      <formula>$H2="Yes"</formula>
     </cfRule>
     <cfRule type="expression" priority="2" dxfId="1">
-      <formula>$G2="No"</formula>
+      <formula>$H2="No"</formula>
     </cfRule>
     <cfRule type="expression" priority="3" dxfId="2">
-      <formula>$G2="Partly"</formula>
+      <formula>$H2="Partly"</formula>
     </cfRule>
     <cfRule type="expression" priority="4" dxfId="3">
-      <formula>$G2="Skipped"</formula>
+      <formula>$H2="Skipped"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="G2:G80" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H2:H80" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Yes,Partly,No,Skipped"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3609,72 +3997,136 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F8" r:id="rId5"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F9" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F10" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F13" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F14" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F15" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F16" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F17" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F18" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F20" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F21" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F22" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F23" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F24" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F25" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F27" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F28" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F29" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F30" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F31" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F32" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F33" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F34" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F35" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F36" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F37" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F38" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F39" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F40" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F41" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F42" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F43" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F44" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F45" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F46" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F47" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F48" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F49" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F50" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F51" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F52" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F53" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F54" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F55" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F56" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F57" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F58" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F59" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F60" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F61" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F62" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F63" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F64" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F65" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F66" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F67" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F68" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F69" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F70" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F71" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F72" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F73" r:id="rId66"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F74" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F75" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F76" r:id="rId69"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F77" r:id="rId70"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F78" r:id="rId71"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F79" r:id="rId72"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F80" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G10" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G11" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F13" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F14" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F15" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G15" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F16" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F17" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F18" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F20" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G21" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F22" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G22" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F23" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G23" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F24" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G24" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F25" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G25" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F27" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G27" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F28" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G28" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F29" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G29" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F30" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G30" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F31" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G31" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F32" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G32" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F33" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G33" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F34" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G34" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F35" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G35" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F36" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G36" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F37" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G37" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F38" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G38" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F39" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G39" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F40" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G40" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F41" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G41" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F42" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G42" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F43" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G43" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F44" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G44" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F45" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G45" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F46" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G46" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F47" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G47" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F48" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G48" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F49" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G49" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F50" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G50" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F51" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G51" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F52" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G52" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F53" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G53" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F54" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G54" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F55" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G55" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F56" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G56" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F57" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G57" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F58" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G58" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F59" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G59" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F60" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G60" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F61" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G61" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F62" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G62" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F63" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G63" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F64" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G64" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F65" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G65" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F66" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G66" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F67" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G67" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F68" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G68" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F69" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G69" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F70" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G70" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F71" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G71" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F72" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G72" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F73" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G73" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F74" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G74" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F75" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G75" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F76" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G76" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F77" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G77" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F78" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G78" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F79" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G79" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F80" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G80" r:id="rId137"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3748,436 +4200,436 @@
       </c>
     </row>
     <row r="2" ht="75" customHeight="1">
-      <c r="A2" s="17" t="n">
+      <c r="A2" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="B2" s="17" t="inlineStr">
+      <c r="B2" s="16" t="inlineStr">
         <is>
           <t>Before Day 1</t>
         </is>
       </c>
-      <c r="C2" s="17" t="inlineStr">
+      <c r="C2" s="16" t="inlineStr">
         <is>
           <t>Setup + where am I today?</t>
         </is>
       </c>
-      <c r="D2" s="17" t="inlineStr">
+      <c r="D2" s="16" t="inlineStr">
         <is>
           <t>A working laptop setup removes the #1 reason people quit in week 1.</t>
         </is>
       </c>
-      <c r="E2" s="17" t="inlineStr">
+      <c r="E2" s="16" t="inlineStr">
         <is>
           <t>Nobody. It's short.</t>
         </is>
       </c>
-      <c r="F2" s="17" t="inlineStr">
+      <c r="F2" s="16" t="inlineStr">
         <is>
           <t>Tools installed, a test cluster ran once, baseline self-check done, one-sentence goal written.</t>
         </is>
       </c>
-      <c r="G2" s="17" t="inlineStr"/>
-      <c r="H2" s="16" t="n"/>
-      <c r="I2" s="16" t="n"/>
+      <c r="G2" s="16" t="inlineStr"/>
+      <c r="H2" s="17" t="n"/>
+      <c r="I2" s="17" t="n"/>
     </row>
     <row r="3" ht="75" customHeight="1">
-      <c r="A3" s="17" t="n">
+      <c r="A3" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="B3" s="17" t="inlineStr">
+      <c r="B3" s="16" t="inlineStr">
         <is>
           <t>1–7</t>
         </is>
       </c>
-      <c r="C3" s="17" t="inlineStr">
+      <c r="C3" s="16" t="inlineStr">
         <is>
           <t>Foundations: Linux, Git, AI as your study partner</t>
         </is>
       </c>
-      <c r="D3" s="17" t="inlineStr">
+      <c r="D3" s="16" t="inlineStr">
         <is>
           <t>Every cloud and DevOps tool assumes you're comfortable in a terminal and with Git. Using AI well makes you learn about 2x faster.</t>
         </is>
       </c>
-      <c r="E3" s="17" t="inlineStr">
+      <c r="E3" s="16" t="inlineStr">
         <is>
           <t>Already comfortable with Linux and Git? Do only Day 5 (AI) and the build day.</t>
         </is>
       </c>
-      <c r="F3" s="17" t="inlineStr">
+      <c r="F3" s="16" t="inlineStr">
         <is>
           <t>Navigate and edit files in a terminal, push a commit to GitHub, and use AI to explain an error safely.</t>
         </is>
       </c>
-      <c r="G3" s="17" t="inlineStr">
+      <c r="G3" s="16" t="inlineStr">
         <is>
           <t>ChatGPT for DevOps: https://www.readyforprod.cloud/courses/chatgpt-for-devops</t>
         </is>
       </c>
-      <c r="H3" s="16" t="n"/>
-      <c r="I3" s="16" t="n"/>
+      <c r="H3" s="17" t="n"/>
+      <c r="I3" s="17" t="n"/>
     </row>
     <row r="4" ht="75" customHeight="1">
-      <c r="A4" s="17" t="n">
+      <c r="A4" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="B4" s="17" t="inlineStr">
+      <c r="B4" s="16" t="inlineStr">
         <is>
           <t>8–14</t>
         </is>
       </c>
-      <c r="C4" s="17" t="inlineStr">
+      <c r="C4" s="16" t="inlineStr">
         <is>
           <t>Docker</t>
         </is>
       </c>
-      <c r="D4" s="17" t="inlineStr">
+      <c r="D4" s="16" t="inlineStr">
         <is>
           <t>Containers are how modern applications are packaged and shipped, everywhere from startups to banks.</t>
         </is>
       </c>
-      <c r="E4" s="17" t="inlineStr">
+      <c r="E4" s="16" t="inlineStr">
         <is>
           <t>You already build and run containers at work.</t>
         </is>
       </c>
-      <c r="F4" s="17" t="inlineStr">
+      <c r="F4" s="16" t="inlineStr">
         <is>
           <t>Write a Dockerfile, build an image, run it with ports and env vars, and run 2 containers together with Compose.</t>
         </is>
       </c>
-      <c r="G4" s="17" t="inlineStr">
+      <c r="G4" s="16" t="inlineStr">
+        <is>
+          <t>ChatGPT for DevOps (lecture: Use ChatGPT for Generating Dockerfile): https://www.readyforprod.cloud/courses/chatgpt-for-devops</t>
+        </is>
+      </c>
+      <c r="H4" s="17" t="n"/>
+      <c r="I4" s="17" t="n"/>
+    </row>
+    <row r="5" ht="75" customHeight="1">
+      <c r="A5" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="B5" s="16" t="inlineStr">
+        <is>
+          <t>15–21</t>
+        </is>
+      </c>
+      <c r="C5" s="16" t="inlineStr">
+        <is>
+          <t>Kubernetes I</t>
+        </is>
+      </c>
+      <c r="D5" s="16" t="inlineStr">
+        <is>
+          <t>Most sizable modern applications run on Kubernetes. It's the common ground of platform, SRE, cloud and DevOps work.</t>
+        </is>
+      </c>
+      <c r="E5" s="16" t="inlineStr">
+        <is>
+          <t>Nobody. This is the core of the challenge.</t>
+        </is>
+      </c>
+      <c r="F5" s="16" t="inlineStr">
+        <is>
+          <t>Run a local cluster, deploy your Week 2 image with a Deployment and Service, scale it, roll it back.</t>
+        </is>
+      </c>
+      <c r="G5" s="16" t="inlineStr">
         <is>
           <t>Hands On Kubernetes: https://www.readyforprod.cloud/courses/hands-on-kubernetes</t>
         </is>
       </c>
-      <c r="H4" s="16" t="n"/>
-      <c r="I4" s="16" t="n"/>
-    </row>
-    <row r="5" ht="75" customHeight="1">
-      <c r="A5" s="17" t="n">
-        <v>3</v>
-      </c>
-      <c r="B5" s="17" t="inlineStr">
-        <is>
-          <t>15–21</t>
-        </is>
-      </c>
-      <c r="C5" s="17" t="inlineStr">
-        <is>
-          <t>Kubernetes I</t>
-        </is>
-      </c>
-      <c r="D5" s="17" t="inlineStr">
-        <is>
-          <t>Most sizable modern applications run on Kubernetes. It's the common ground of platform, SRE, cloud and DevOps work.</t>
-        </is>
-      </c>
-      <c r="E5" s="17" t="inlineStr">
-        <is>
-          <t>Nobody. This is the core of the challenge.</t>
-        </is>
-      </c>
-      <c r="F5" s="17" t="inlineStr">
-        <is>
-          <t>Run a local cluster, deploy your Week 2 image with a Deployment and Service, scale it, roll it back.</t>
-        </is>
-      </c>
-      <c r="G5" s="17" t="inlineStr">
-        <is>
-          <t>Hands On Kubernetes: https://www.readyforprod.cloud/courses/hands-on-kubernetes</t>
-        </is>
-      </c>
-      <c r="H5" s="16" t="n"/>
-      <c r="I5" s="16" t="n"/>
+      <c r="H5" s="17" t="n"/>
+      <c r="I5" s="17" t="n"/>
     </row>
     <row r="6" ht="75" customHeight="1">
-      <c r="A6" s="17" t="n">
+      <c r="A6" s="16" t="n">
         <v>4</v>
       </c>
-      <c r="B6" s="17" t="inlineStr">
+      <c r="B6" s="16" t="inlineStr">
         <is>
           <t>22–28</t>
         </is>
       </c>
-      <c r="C6" s="17" t="inlineStr">
+      <c r="C6" s="16" t="inlineStr">
         <is>
           <t>Kubernetes II: production basics</t>
         </is>
       </c>
-      <c r="D6" s="17" t="inlineStr">
+      <c r="D6" s="16" t="inlineStr">
         <is>
           <t>The difference between 'it runs' and 'it's production-ready': config, secrets, health checks, resources, storage.</t>
         </is>
       </c>
-      <c r="E6" s="17" t="inlineStr">
+      <c r="E6" s="16" t="inlineStr">
         <is>
           <t>Nobody.</t>
         </is>
       </c>
-      <c r="F6" s="17" t="inlineStr">
+      <c r="F6" s="16" t="inlineStr">
         <is>
           <t>Add ConfigMap/Secret, probes and requests/limits to your app; know when to use a Job, CronJob or Deployment; use a PVC; solve the 6 Broken Kubernetes exercises.</t>
         </is>
       </c>
-      <c r="G6" s="17" t="inlineStr">
+      <c r="G6" s="16" t="inlineStr">
         <is>
           <t>k8s Production Readiness: https://www.readyforprod.cloud/courses/k8s-production-readiness</t>
         </is>
       </c>
-      <c r="H6" s="16" t="n"/>
-      <c r="I6" s="16" t="n"/>
+      <c r="H6" s="17" t="n"/>
+      <c r="I6" s="17" t="n"/>
     </row>
     <row r="7" ht="75" customHeight="1">
-      <c r="A7" s="17" t="n">
+      <c r="A7" s="16" t="n">
         <v>5</v>
       </c>
-      <c r="B7" s="17" t="inlineStr">
+      <c r="B7" s="16" t="inlineStr">
         <is>
           <t>29–35</t>
         </is>
       </c>
-      <c r="C7" s="17" t="inlineStr">
+      <c r="C7" s="16" t="inlineStr">
         <is>
           <t>Checkpoint 1: projects + self-check</t>
         </is>
       </c>
-      <c r="D7" s="17" t="inlineStr">
+      <c r="D7" s="16" t="inlineStr">
         <is>
           <t>Proof you can do it, not just watch it. This becomes your first portfolio piece.</t>
         </is>
       </c>
-      <c r="E7" s="17" t="inlineStr">
+      <c r="E7" s="16" t="inlineStr">
         <is>
           <t>Nobody.</t>
         </is>
       </c>
-      <c r="F7" s="17" t="inlineStr">
+      <c r="F7" s="16" t="inlineStr">
         <is>
           <t>Finish Checkpoint 1 project, fix the broken YAML exercise, complete the Week 5 self-check.</t>
         </is>
       </c>
-      <c r="G7" s="17" t="inlineStr"/>
-      <c r="H7" s="16" t="n"/>
-      <c r="I7" s="16" t="n"/>
+      <c r="G7" s="16" t="inlineStr"/>
+      <c r="H7" s="17" t="n"/>
+      <c r="I7" s="17" t="n"/>
     </row>
     <row r="8" ht="75" customHeight="1">
-      <c r="A8" s="17" t="n">
+      <c r="A8" s="16" t="n">
         <v>6</v>
       </c>
-      <c r="B8" s="17" t="inlineStr">
+      <c r="B8" s="16" t="inlineStr">
         <is>
           <t>36–42</t>
         </is>
       </c>
-      <c r="C8" s="17" t="inlineStr">
+      <c r="C8" s="16" t="inlineStr">
         <is>
           <t>CI/CD with GitHub Actions</t>
         </is>
       </c>
-      <c r="D8" s="17" t="inlineStr">
+      <c r="D8" s="16" t="inlineStr">
         <is>
           <t>Automating build, test and deploy is the heart of DevOps and platform work.</t>
         </is>
       </c>
-      <c r="E8" s="17" t="inlineStr">
+      <c r="E8" s="16" t="inlineStr">
         <is>
           <t>You already maintain pipelines at work.</t>
         </is>
       </c>
-      <c r="F8" s="17" t="inlineStr">
+      <c r="F8" s="16" t="inlineStr">
         <is>
           <t>A pipeline that builds and tests on every push and publishes your container image.</t>
         </is>
       </c>
-      <c r="G8" s="17" t="inlineStr">
+      <c r="G8" s="16" t="inlineStr">
         <is>
           <t>Learning GitHub Actions for DevOps CI/CD: https://www.readyforprod.cloud/courses/learning-github-actions</t>
         </is>
       </c>
-      <c r="H8" s="16" t="n"/>
-      <c r="I8" s="16" t="n"/>
+      <c r="H8" s="17" t="n"/>
+      <c r="I8" s="17" t="n"/>
     </row>
     <row r="9" ht="75" customHeight="1">
-      <c r="A9" s="17" t="n">
+      <c r="A9" s="16" t="n">
         <v>7</v>
       </c>
-      <c r="B9" s="17" t="inlineStr">
+      <c r="B9" s="16" t="inlineStr">
         <is>
           <t>43–49</t>
         </is>
       </c>
-      <c r="C9" s="17" t="inlineStr">
+      <c r="C9" s="16" t="inlineStr">
         <is>
           <t>Cloud for admins (Azure)</t>
         </is>
       </c>
-      <c r="D9" s="17" t="inlineStr">
+      <c r="D9" s="16" t="inlineStr">
         <is>
           <t>Admin jobs are moving to the cloud. The concepts (networks, identity, resource groups) carry over to every cloud.</t>
         </is>
       </c>
-      <c r="E9" s="17" t="inlineStr">
+      <c r="E9" s="16" t="inlineStr">
         <is>
           <t>Committed to AWS or GCP? Learn the same concepts there instead.</t>
         </is>
       </c>
-      <c r="F9" s="17" t="inlineStr">
+      <c r="F9" s="16" t="inlineStr">
         <is>
           <t>Create and clean up resources, understand VNets and identities (Managed Identity vs Service Principal).</t>
         </is>
       </c>
-      <c r="G9" s="17" t="inlineStr">
+      <c r="G9" s="16" t="inlineStr">
         <is>
           <t>AZ-900 Quick Prep: https://www.readyforprod.cloud/courses/az900-azure-fundamentals · Learning Microsoft Azure: https://www.readyforprod.cloud/courses/learning-microsoft-azure</t>
         </is>
       </c>
-      <c r="H9" s="16" t="n"/>
-      <c r="I9" s="16" t="n"/>
+      <c r="H9" s="17" t="n"/>
+      <c r="I9" s="17" t="n"/>
     </row>
     <row r="10" ht="75" customHeight="1">
-      <c r="A10" s="17" t="n">
+      <c r="A10" s="16" t="n">
         <v>8</v>
       </c>
-      <c r="B10" s="17" t="inlineStr">
+      <c r="B10" s="16" t="inlineStr">
         <is>
           <t>50–56</t>
         </is>
       </c>
-      <c r="C10" s="17" t="inlineStr">
+      <c r="C10" s="16" t="inlineStr">
         <is>
           <t>Terraform (infrastructure as code)</t>
         </is>
       </c>
-      <c r="D10" s="17" t="inlineStr">
+      <c r="D10" s="16" t="inlineStr">
         <is>
           <t>The modern way enterprises create infrastructure reliably, predictably and repeatably.</t>
         </is>
       </c>
-      <c r="E10" s="17" t="inlineStr">
+      <c r="E10" s="16" t="inlineStr">
         <is>
           <t>Truly never going to touch infrastructure? Try Day 50. If it's honestly not for you, skip to Week 9.</t>
         </is>
       </c>
-      <c r="F10" s="17" t="inlineStr">
+      <c r="F10" s="16" t="inlineStr">
         <is>
           <t>Write, plan, apply and destroy infrastructure with Terraform; understand state and variables.</t>
         </is>
       </c>
-      <c r="G10" s="17" t="inlineStr">
+      <c r="G10" s="16" t="inlineStr">
         <is>
           <t>Terraform For GenAI DevOps Engineer: https://www.readyforprod.cloud/courses/terraform-for-devops</t>
         </is>
       </c>
-      <c r="H10" s="16" t="n"/>
-      <c r="I10" s="16" t="n"/>
+      <c r="H10" s="17" t="n"/>
+      <c r="I10" s="17" t="n"/>
     </row>
     <row r="11" ht="75" customHeight="1">
-      <c r="A11" s="17" t="n">
+      <c r="A11" s="16" t="n">
         <v>9</v>
       </c>
-      <c r="B11" s="17" t="inlineStr">
+      <c r="B11" s="16" t="inlineStr">
         <is>
           <t>57–63</t>
         </is>
       </c>
-      <c r="C11" s="17" t="inlineStr">
+      <c r="C11" s="16" t="inlineStr">
         <is>
           <t>Checkpoint 2: end-to-end project</t>
         </is>
       </c>
-      <c r="D11" s="17" t="inlineStr">
+      <c r="D11" s="16" t="inlineStr">
         <is>
           <t>End-to-end proof for your CV: pipeline, infrastructure and app working together.</t>
         </is>
       </c>
-      <c r="E11" s="17" t="inlineStr">
+      <c r="E11" s="16" t="inlineStr">
         <is>
           <t>Nobody.</t>
         </is>
       </c>
-      <c r="F11" s="17" t="inlineStr">
+      <c r="F11" s="16" t="inlineStr">
         <is>
           <t>Finish Checkpoint 2 project and the 'find the problems in this pipeline' exercise; Week 9 self-check.</t>
         </is>
       </c>
-      <c r="G11" s="17" t="inlineStr"/>
-      <c r="H11" s="16" t="n"/>
-      <c r="I11" s="16" t="n"/>
+      <c r="G11" s="16" t="inlineStr"/>
+      <c r="H11" s="17" t="n"/>
+      <c r="I11" s="17" t="n"/>
     </row>
     <row r="12" ht="75" customHeight="1">
-      <c r="A12" s="17" t="n">
+      <c r="A12" s="16" t="n">
         <v>10</v>
       </c>
-      <c r="B12" s="17" t="inlineStr">
+      <c r="B12" s="16" t="inlineStr">
         <is>
           <t>64–70</t>
         </is>
       </c>
-      <c r="C12" s="17" t="inlineStr">
+      <c r="C12" s="16" t="inlineStr">
         <is>
           <t>AI in DevOps and SRE</t>
         </is>
       </c>
-      <c r="D12" s="17" t="inlineStr">
+      <c r="D12" s="16" t="inlineStr">
         <is>
           <t>Where the market is heading. Use AI to troubleshoot faster, and learn to run AI apps as just another workload.</t>
         </is>
       </c>
-      <c r="E12" s="17" t="inlineStr">
+      <c r="E12" s="16" t="inlineStr">
         <is>
           <t>Nobody.</t>
         </is>
       </c>
-      <c r="F12" s="17" t="inlineStr">
+      <c r="F12" s="16" t="inlineStr">
         <is>
           <t>Troubleshoot with AI safely, understand logs vs metrics, run a small AI app as a workload.</t>
         </is>
       </c>
-      <c r="G12" s="17" t="inlineStr">
+      <c r="G12" s="16" t="inlineStr">
         <is>
           <t>ChatGPT for DevOps: https://www.readyforprod.cloud/courses/chatgpt-for-devops · n8n Masterclass: https://www.readyforprod.cloud/courses/n8n-masterclass</t>
         </is>
       </c>
-      <c r="H12" s="16" t="n"/>
-      <c r="I12" s="16" t="n"/>
+      <c r="H12" s="17" t="n"/>
+      <c r="I12" s="17" t="n"/>
     </row>
     <row r="13" ht="75" customHeight="1">
-      <c r="A13" s="17" t="n">
+      <c r="A13" s="16" t="n">
         <v>11</v>
       </c>
-      <c r="B13" s="17" t="inlineStr">
+      <c r="B13" s="16" t="inlineStr">
         <is>
           <t>71–75</t>
         </is>
       </c>
-      <c r="C13" s="17" t="inlineStr">
+      <c r="C13" s="16" t="inlineStr">
         <is>
           <t>Capstone + pick your path</t>
         </is>
       </c>
-      <c r="D13" s="17" t="inlineStr">
+      <c r="D13" s="16" t="inlineStr">
         <is>
           <t>Turn 75 days into a story you can tell in an interview, and choose where to go deep next.</t>
         </is>
       </c>
-      <c r="E13" s="17" t="inlineStr">
+      <c r="E13" s="16" t="inlineStr">
         <is>
           <t>Nobody.</t>
         </is>
       </c>
-      <c r="F13" s="17" t="inlineStr">
+      <c r="F13" s="16" t="inlineStr">
         <is>
           <t>Capstone done, final self-check, 3 CV bullets written, next path chosen.</t>
         </is>
       </c>
-      <c r="G13" s="17" t="inlineStr">
+      <c r="G13" s="16" t="inlineStr">
         <is>
           <t>The whole path, with your challenge price: https://www.readyforprod.cloud/bundles/ai-enabled-devops-sre?coupon=UPGRADE75</t>
         </is>
       </c>
-      <c r="H13" s="16" t="n"/>
-      <c r="I13" s="16" t="n"/>
+      <c r="H13" s="17" t="n"/>
+      <c r="I13" s="17" t="n"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="H2:H13">
@@ -4253,223 +4705,223 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="17" t="n">
+      <c r="A2" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="17" t="inlineStr">
+      <c r="B2" s="16" t="inlineStr">
         <is>
           <t>move around folders and edit files in a Linux terminal?</t>
         </is>
       </c>
-      <c r="C2" s="16" t="n"/>
-      <c r="D2" s="16" t="n"/>
-      <c r="E2" s="16" t="n"/>
-      <c r="F2" s="16" t="n"/>
+      <c r="C2" s="17" t="n"/>
+      <c r="D2" s="17" t="n"/>
+      <c r="E2" s="17" t="n"/>
+      <c r="F2" s="17" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="17" t="n">
+      <c r="A3" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="17" t="inlineStr">
+      <c r="B3" s="16" t="inlineStr">
         <is>
           <t>clone a Git repo, commit and push a change?</t>
         </is>
       </c>
-      <c r="C3" s="16" t="n"/>
-      <c r="D3" s="16" t="n"/>
-      <c r="E3" s="16" t="n"/>
-      <c r="F3" s="16" t="n"/>
+      <c r="C3" s="17" t="n"/>
+      <c r="D3" s="17" t="n"/>
+      <c r="E3" s="17" t="n"/>
+      <c r="F3" s="17" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="17" t="n">
+      <c r="A4" s="16" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="17" t="inlineStr">
+      <c r="B4" s="16" t="inlineStr">
         <is>
           <t>explain what a container is and how it differs from a VM?</t>
         </is>
       </c>
-      <c r="C4" s="16" t="n"/>
-      <c r="D4" s="16" t="n"/>
-      <c r="E4" s="16" t="n"/>
-      <c r="F4" s="16" t="n"/>
+      <c r="C4" s="17" t="n"/>
+      <c r="D4" s="17" t="n"/>
+      <c r="E4" s="17" t="n"/>
+      <c r="F4" s="17" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="17" t="n">
+      <c r="A5" s="16" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="17" t="inlineStr">
+      <c r="B5" s="16" t="inlineStr">
         <is>
           <t>explain what Kubernetes does, to a friend?</t>
         </is>
       </c>
-      <c r="C5" s="16" t="n"/>
-      <c r="D5" s="16" t="n"/>
-      <c r="E5" s="16" t="n"/>
-      <c r="F5" s="16" t="n"/>
+      <c r="C5" s="17" t="n"/>
+      <c r="D5" s="17" t="n"/>
+      <c r="E5" s="17" t="n"/>
+      <c r="F5" s="17" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="17" t="n">
+      <c r="A6" s="16" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="17" t="inlineStr">
+      <c r="B6" s="16" t="inlineStr">
         <is>
           <t>deploy an app built from a Dockerfile to Kubernetes?</t>
         </is>
       </c>
-      <c r="C6" s="16" t="n"/>
-      <c r="D6" s="16" t="n"/>
-      <c r="E6" s="16" t="n"/>
-      <c r="F6" s="16" t="n"/>
+      <c r="C6" s="17" t="n"/>
+      <c r="D6" s="17" t="n"/>
+      <c r="E6" s="17" t="n"/>
+      <c r="F6" s="17" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="17" t="n">
+      <c r="A7" s="16" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="17" t="inlineStr">
+      <c r="B7" s="16" t="inlineStr">
         <is>
           <t>explain when to use a Job, a CronJob or a Deployment?</t>
         </is>
       </c>
-      <c r="C7" s="16" t="n"/>
-      <c r="D7" s="16" t="n"/>
-      <c r="E7" s="16" t="n"/>
-      <c r="F7" s="16" t="n"/>
+      <c r="C7" s="17" t="n"/>
+      <c r="D7" s="17" t="n"/>
+      <c r="E7" s="17" t="n"/>
+      <c r="F7" s="17" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="17" t="n">
+      <c r="A8" s="16" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="17" t="inlineStr">
+      <c r="B8" s="16" t="inlineStr">
         <is>
           <t>use a PersistentVolumeClaim comfortably?</t>
         </is>
       </c>
-      <c r="C8" s="16" t="n"/>
-      <c r="D8" s="16" t="n"/>
-      <c r="E8" s="16" t="n"/>
-      <c r="F8" s="16" t="n"/>
+      <c r="C8" s="17" t="n"/>
+      <c r="D8" s="17" t="n"/>
+      <c r="E8" s="17" t="n"/>
+      <c r="F8" s="17" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="17" t="n">
+      <c r="A9" s="16" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="17" t="inlineStr">
+      <c r="B9" s="16" t="inlineStr">
         <is>
           <t>say why a Kubernetes YAML is NOT production-ready (probes, limits, secrets, image tags)?</t>
         </is>
       </c>
-      <c r="C9" s="16" t="n"/>
-      <c r="D9" s="16" t="n"/>
-      <c r="E9" s="16" t="n"/>
-      <c r="F9" s="16" t="n"/>
+      <c r="C9" s="17" t="n"/>
+      <c r="D9" s="17" t="n"/>
+      <c r="E9" s="17" t="n"/>
+      <c r="F9" s="17" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="17" t="n">
+      <c r="A10" s="16" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="17" t="inlineStr">
+      <c r="B10" s="16" t="inlineStr">
         <is>
           <t>build a CI/CD pipeline that builds and tests on every push?</t>
         </is>
       </c>
-      <c r="C10" s="16" t="n"/>
-      <c r="D10" s="16" t="n"/>
-      <c r="E10" s="16" t="n"/>
-      <c r="F10" s="16" t="n"/>
+      <c r="C10" s="17" t="n"/>
+      <c r="D10" s="17" t="n"/>
+      <c r="E10" s="17" t="n"/>
+      <c r="F10" s="17" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="17" t="n">
+      <c r="A11" s="16" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="17" t="inlineStr">
+      <c r="B11" s="16" t="inlineStr">
         <is>
           <t>create something in a cloud and clean it up again?</t>
         </is>
       </c>
-      <c r="C11" s="16" t="n"/>
-      <c r="D11" s="16" t="n"/>
-      <c r="E11" s="16" t="n"/>
-      <c r="F11" s="16" t="n"/>
+      <c r="C11" s="17" t="n"/>
+      <c r="D11" s="17" t="n"/>
+      <c r="E11" s="17" t="n"/>
+      <c r="F11" s="17" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="17" t="n">
+      <c r="A12" s="16" t="n">
         <v>11</v>
       </c>
-      <c r="B12" s="17" t="inlineStr">
+      <c r="B12" s="16" t="inlineStr">
         <is>
           <t>explain what infrastructure as code means, and use Terraform plan/apply?</t>
         </is>
       </c>
-      <c r="C12" s="16" t="n"/>
-      <c r="D12" s="16" t="n"/>
-      <c r="E12" s="16" t="n"/>
-      <c r="F12" s="16" t="n"/>
+      <c r="C12" s="17" t="n"/>
+      <c r="D12" s="17" t="n"/>
+      <c r="E12" s="17" t="n"/>
+      <c r="F12" s="17" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="17" t="n">
+      <c r="A13" s="16" t="n">
         <v>12</v>
       </c>
-      <c r="B13" s="17" t="inlineStr">
+      <c r="B13" s="16" t="inlineStr">
         <is>
           <t>use an AI assistant at work safely, at least once a week?</t>
         </is>
       </c>
-      <c r="C13" s="16" t="n"/>
-      <c r="D13" s="16" t="n"/>
-      <c r="E13" s="16" t="n"/>
-      <c r="F13" s="16" t="n"/>
+      <c r="C13" s="17" t="n"/>
+      <c r="D13" s="17" t="n"/>
+      <c r="E13" s="17" t="n"/>
+      <c r="F13" s="17" t="n"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr"/>
-      <c r="B15" s="18" t="inlineStr">
+      <c r="B15" s="19" t="inlineStr">
         <is>
           <t>My level (count of Yes)</t>
         </is>
       </c>
-      <c r="C15" s="18">
+      <c r="C15" s="19">
         <f>COUNTIF(C2:C13,"Yes")</f>
         <v/>
       </c>
-      <c r="D15" s="18">
+      <c r="D15" s="19">
         <f>COUNTIF(D2:D13,"Yes")</f>
         <v/>
       </c>
-      <c r="E15" s="18">
+      <c r="E15" s="19">
         <f>COUNTIF(E2:E13,"Yes")</f>
         <v/>
       </c>
-      <c r="F15" s="18">
+      <c r="F15" s="19">
         <f>COUNTIF(F2:F13,"Yes")</f>
         <v/>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr"/>
-      <c r="B16" s="18" t="inlineStr">
+      <c r="B16" s="19" t="inlineStr">
         <is>
           <t>Level</t>
         </is>
       </c>
-      <c r="C16" s="18">
+      <c r="C16" s="19">
         <f>IF(C15&gt;=9,"Intermediate",IF(C15&gt;=5,"Working","Starter"))</f>
         <v/>
       </c>
-      <c r="D16" s="18">
+      <c r="D16" s="19">
         <f>IF(D15&gt;=9,"Intermediate",IF(D15&gt;=5,"Working","Starter"))</f>
         <v/>
       </c>
-      <c r="E16" s="18">
+      <c r="E16" s="19">
         <f>IF(E15&gt;=9,"Intermediate",IF(E15&gt;=5,"Working","Starter"))</f>
         <v/>
       </c>
-      <c r="F16" s="18">
+      <c r="F16" s="19">
         <f>IF(F15&gt;=9,"Intermediate",IF(F15&gt;=5,"Working","Starter"))</f>
         <v/>
       </c>
     </row>
     <row r="18">
-      <c r="B18" s="19" t="inlineStr">
+      <c r="B18" s="20" t="inlineStr">
         <is>
           <t>Levels: 0–4 Yes = Starter · 5–8 = Working · 9–12 = Intermediate. Nobody is an 'expert'; everyone keeps exploring.</t>
         </is>
@@ -4573,61 +5025,61 @@
       </c>
     </row>
     <row r="2" ht="60" customHeight="1">
-      <c r="A2" s="20" t="inlineStr">
+      <c r="A2" s="21" t="inlineStr">
         <is>
           <t>Checkpoint 1: app on Kubernetes</t>
         </is>
       </c>
-      <c r="B2" s="17" t="inlineStr">
+      <c r="B2" s="16" t="inlineStr">
         <is>
           <t>Week 5</t>
         </is>
       </c>
-      <c r="C2" s="17" t="inlineStr">
+      <c r="C2" s="16" t="inlineStr">
         <is>
           <t>Run the 2-tier Notes app (Flask + Redis) on kind the production-ready way: namespace, Secret, ConfigMap, probes, limits, 2 replicas, and notes that survive a Redis restart (PVC).</t>
         </is>
       </c>
-      <c r="D2" s="16" t="n"/>
-      <c r="E2" s="16" t="n"/>
+      <c r="D2" s="17" t="n"/>
+      <c r="E2" s="17" t="n"/>
     </row>
     <row r="3" ht="60" customHeight="1">
-      <c r="A3" s="20" t="inlineStr">
+      <c r="A3" s="21" t="inlineStr">
         <is>
           <t>Checkpoint 2: end to end</t>
         </is>
       </c>
-      <c r="B3" s="17" t="inlineStr">
+      <c r="B3" s="16" t="inlineStr">
         <is>
           <t>Week 9</t>
         </is>
       </c>
-      <c r="C3" s="17" t="inlineStr">
+      <c r="C3" s="16" t="inlineStr">
         <is>
           <t>Every push to main tests, builds (SHA-tagged image) and deploys the Notes app onto a platform Terraform creates, with a smoke test that turns the pipeline red if the app is broken. Plus the flawed-pipeline review.</t>
         </is>
       </c>
-      <c r="D3" s="16" t="n"/>
-      <c r="E3" s="16" t="n"/>
+      <c r="D3" s="17" t="n"/>
+      <c r="E3" s="17" t="n"/>
     </row>
     <row r="4" ht="60" customHeight="1">
-      <c r="A4" s="20" t="inlineStr">
+      <c r="A4" s="21" t="inlineStr">
         <is>
           <t>Capstone: AI app to production</t>
         </is>
       </c>
-      <c r="B4" s="17" t="inlineStr">
+      <c r="B4" s="16" t="inlineStr">
         <is>
           <t>Week 11</t>
         </is>
       </c>
-      <c r="C4" s="17" t="inlineStr">
+      <c r="C4" s="16" t="inlineStr">
         <is>
           <t>Run the Error Explainer AI app like any production workload: secrets never reach the LLM, health checks, metrics, timeouts, a runbook. Then pick your path and write 3 CV bullets.</t>
         </is>
       </c>
-      <c r="D4" s="16" t="n"/>
-      <c r="E4" s="16" t="n"/>
+      <c r="D4" s="17" t="n"/>
+      <c r="E4" s="17" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="1">

</xml_diff>